<commit_message>
Aplicar el Manual de Identidad de Rebis al cash-flow
Presentación del libro según el manual: wordmark negro en la esquina superior
derecha de cada hoja con su área de protección, titulares por debajo del
logotipo, tipografía Arial Regular y Bold —la fuente de sistema que el manual
designa para entornos técnicos y administrativos, donde Poppins no está
disponible—, paleta principal de negro y tonos arquitectónicos, y Roble
Natural reservado como único acento sobre la rentabilidad final y la URL.

Los datos de entrada pasan del azul de convención financiera a un fondo
cerámica, que sí pertenece a la paleta. Se corrige la escritura del nombre,
que el manual exige con mayúscula inicial y minúsculas. Cada hoja cierra con
la tagline y rebis.com alineada a la derecha.

Las cifras no cambian.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3Mnw54UTuPQAtnGvXf7kT
</commit_message>
<xml_diff>
--- a/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
+++ b/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
@@ -18,11 +18,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;;(#,##0 &quot;€&quot;);- "/>
-    <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;;(#,##0.00 &quot;€&quot;);- "/>
-    <numFmt numFmtId="166" formatCode="0.00&quot;%&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;;(#,##0 &quot;€&quot;);—"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;;(#,##0.00 &quot;€&quot;);—"/>
+    <numFmt numFmtId="166" formatCode="0.00&quot; %&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,34 +32,24 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF808282"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="FF000000"/>
-      <sz val="16"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="Arial"/>
       <color rgb="FF515150"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="FF0000FF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -72,20 +62,43 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FF808282"/>
-      <sz val="8"/>
+      <sz val="7.5"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF515150"/>
-      <sz val="9"/>
+      <color rgb="FF808282"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFB59169"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <color rgb="FF515150"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FFB59169"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -94,7 +107,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF515150"/>
+        <fgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD7D1CA"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,63 +153,71 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -267,6 +293,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>104775</colOff>
+      <row>0</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="1143000" cy="438150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>104775</colOff>
+      <row>0</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="1143000" cy="438150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -558,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C95"/>
+  <dimension ref="A3:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -566,973 +652,984 @@
     <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>REBIS · DESARROLLOS INMOBILIARIOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cash-Flow del Inversor  ·  Opción 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Apartamento calle Ruiz Jiménez 3, Madrid  ·  La operación se canaliza a través de la sociedad de Rebis; el Inversor entra mediante préstamo participativo  ·  Escenario conservador</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="1" ht="52" customHeight="1"/>
+    <row r="2" ht="8" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Cash-Flow del Inversor · Opción 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Apartamento calle Ruiz Jiménez 3, Madrid.  La operación se canaliza a través de la sociedad de Rebis y el Inversor entra mediante préstamo participativo.  Escenario conservador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="6" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>RESUMEN DE COMPRA Y VENTA</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Precio de compra</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="8" t="n">
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="n">
         <v>1500000</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>M2 construidos</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="9" t="n">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="8" t="n">
         <v>176</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Precio del m2 de compra</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="10">
-        <f>C7/C8</f>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="11">
+        <f>C8/C9</f>
         <v>8522.7272727273</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Precio del m2 de venta</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="11" t="n">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="12" t="n">
         <v>14200</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Precio de venta estimado</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="13">
-        <f>C10*C8</f>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="14">
+        <f>C11*C9</f>
         <v>2499200</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>COSTES  ·  IMPORTES CON IVA INCLUIDO</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>ACTUACIÓN</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>CONCEPTO</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>IMPORTE</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Adquisición</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Comisión inmobiliaria</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>45375</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="16" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="n"/>
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Honorarios legales por análisis de documentación</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C17" s="18" t="n">
         <v>1270.5</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="16" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="9" t="n"/>
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>ITP · IVA · AJD</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C18" s="18" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="n"/>
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Notaría</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C19" s="18" t="n">
         <v>2700</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="16" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Gestoría</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C20" s="18" t="n">
         <v>494</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="16" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Registro de la propiedad</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C21" s="18" t="n">
         <v>1600</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="n"/>
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>IBI y tasas de basuras, proporcional 2026</t>
         </is>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C22" s="18" t="n">
         <v>875</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Total adquisición</t>
         </is>
       </c>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="20">
-        <f>SUM(C15:C21)</f>
+      <c r="B23" s="20" t="n"/>
+      <c r="C23" s="21">
+        <f>SUM(C16:C22)</f>
         <v>82314.5</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Financiación bancaria</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Tasación</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C24" s="18" t="n">
         <v>605</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="16" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="n"/>
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Pago otorgamiento de hipoteca (AJD)</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C25" s="18" t="n">
         <v>9000</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="16" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="9" t="n"/>
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Comisión por otorgamiento de hipoteca</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C26" s="18" t="n">
         <v>2475</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="16" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="n"/>
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>Contribución especial Fundación CaixaBank</t>
         </is>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C27" s="18" t="n">
         <v>1200</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>Pignoración (fondo recuperable, ver nota 1)</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="n">
+    <row r="28">
+      <c r="A28" s="9" t="n"/>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Pignoración · fondo recuperable, ver nota 1</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="n">
         <v>38000</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="16" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="9" t="n"/>
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Gastos de hipoteca</t>
         </is>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C29" s="18" t="n">
         <v>35062.5</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="16" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="n"/>
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Seguro de responsabilidad civil</t>
         </is>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C30" s="18" t="n">
         <v>649.51</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="16" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="n"/>
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Notaría</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C31" s="18" t="n">
         <v>2000</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="16" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="n"/>
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Gestoría</t>
         </is>
       </c>
-      <c r="C31" s="17" t="n">
+      <c r="C32" s="18" t="n">
         <v>494</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="16" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>Registro de la propiedad</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C33" s="18" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Total financiación bancaria</t>
         </is>
       </c>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="20">
-        <f>SUM(C23:C32)</f>
+      <c r="B34" s="20" t="n"/>
+      <c r="C34" s="21">
+        <f>SUM(C24:C33)</f>
         <v>90386.01</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>Reforma</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>Seguro de incendio</t>
         </is>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C35" s="18" t="n">
         <v>703.9400000000001</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="16" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="9" t="n"/>
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>Asamblea para aprobación de reformas en áreas comunes</t>
         </is>
       </c>
-      <c r="C35" s="17" t="n">
+      <c r="C36" s="18" t="n">
         <v>150</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="16" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>Obra</t>
         </is>
       </c>
-      <c r="C36" s="17" t="n">
+      <c r="C37" s="18" t="n">
         <v>325000</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="16" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="9" t="n"/>
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>Muebles</t>
         </is>
       </c>
-      <c r="C37" s="17" t="n">
+      <c r="C38" s="18" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="16" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Imprevistos</t>
         </is>
       </c>
-      <c r="C38" s="17" t="n">
+      <c r="C39" s="18" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="16" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>Honorarios de interiorismo y arquitectura</t>
         </is>
       </c>
-      <c r="C39" s="17" t="n">
+      <c r="C40" s="18" t="n">
         <v>6500</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="16" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="n"/>
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>Impuestos corrientes durante la ejecución de obra</t>
         </is>
       </c>
-      <c r="C40" s="17" t="n">
+      <c r="C41" s="18" t="n">
         <v>5300</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="18" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>Total reforma</t>
         </is>
       </c>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="20">
-        <f>SUM(C34:C40)</f>
+      <c r="B42" s="20" t="n"/>
+      <c r="C42" s="21">
+        <f>SUM(C35:C41)</f>
         <v>382653.94</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Venta</t>
         </is>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B43" s="17" t="inlineStr">
         <is>
           <t>Fotografía y afines</t>
         </is>
       </c>
-      <c r="C42" s="17" t="n">
+      <c r="C43" s="18" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="16" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="9" t="n"/>
+      <c r="B44" s="17" t="inlineStr">
         <is>
           <t>IBI y tasas de basuras, proporcional 2027</t>
         </is>
       </c>
-      <c r="C43" s="17" t="n">
+      <c r="C44" s="18" t="n">
         <v>400</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="16" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="9" t="n"/>
+      <c r="B45" s="17" t="inlineStr">
         <is>
           <t>Comisión inmobiliaria</t>
         </is>
       </c>
-      <c r="C44" s="17">
-        <f>ROUND($C$11*0.0363,2)</f>
+      <c r="C45" s="18">
+        <f>ROUND($C$12*0.0363,2)</f>
         <v>90720.96</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="16" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="9" t="n"/>
+      <c r="B46" s="17" t="inlineStr">
         <is>
           <t>Plusvalía municipal</t>
         </is>
       </c>
-      <c r="C45" s="17" t="n">
+      <c r="C46" s="18" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="18" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
         <is>
           <t>Total venta</t>
         </is>
       </c>
-      <c r="B46" s="19" t="n"/>
-      <c r="C46" s="20">
-        <f>SUM(C42:C45)</f>
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="21">
+        <f>SUM(C43:C46)</f>
         <v>107020.96</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
         <is>
           <t>Financiación por venta</t>
         </is>
       </c>
-      <c r="B47" s="16" t="inlineStr">
+      <c r="B48" s="17" t="inlineStr">
         <is>
           <t>Comisión por cancelación de hipoteca</t>
         </is>
       </c>
-      <c r="C47" s="17" t="n">
+      <c r="C48" s="18" t="n">
         <v>1237.5</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="16" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="9" t="n"/>
+      <c r="B49" s="17" t="inlineStr">
         <is>
           <t>Gestoría por cancelación de hipoteca</t>
         </is>
       </c>
-      <c r="C48" s="17" t="n">
+      <c r="C49" s="18" t="n">
         <v>494</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="16" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="9" t="n"/>
+      <c r="B50" s="17" t="inlineStr">
         <is>
           <t>Registro de la propiedad por cancelación</t>
         </is>
       </c>
-      <c r="C49" s="17" t="n">
+      <c r="C50" s="18" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="18" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Total financiación por venta</t>
         </is>
       </c>
-      <c r="B50" s="19" t="n"/>
-      <c r="C50" s="20">
-        <f>SUM(C47:C49)</f>
+      <c r="B51" s="20" t="n"/>
+      <c r="C51" s="21">
+        <f>SUM(C48:C50)</f>
         <v>2731.5</v>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  (SIN GASTOS DE VENTA NI DE FINANCIACIÓN)</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="53" ht="17" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  ·  SIN GASTOS DE VENTA NI DE FINANCIACIÓN</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>Compra del apartamento</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="17">
-        <f>$C$7</f>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="18">
+        <f>$C$8</f>
         <v>1500000</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>Gastos derivados de la adquisición</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="17">
-        <f>C22</f>
+      <c r="B55" s="10" t="n"/>
+      <c r="C55" s="18">
+        <f>C23</f>
         <v>82314.5</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Gastos de reforma</t>
         </is>
       </c>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="17">
-        <f>C41</f>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="18">
+        <f>C42</f>
         <v>382653.94</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>Fotografía y afines</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n"/>
-      <c r="C56" s="17" t="n">
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="18" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="21" t="inlineStr">
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Capital necesario</t>
         </is>
       </c>
-      <c r="B57" s="22" t="n"/>
-      <c r="C57" s="23">
-        <f>SUM(C53:C56)</f>
+      <c r="B58" s="23" t="n"/>
+      <c r="C58" s="24">
+        <f>SUM(C54:C57)</f>
         <v>1965868.44</v>
       </c>
     </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="60" ht="17" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>APORTES DE CAPITAL</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n"/>
-      <c r="C59" s="5" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>Aporte de capital bancario · Rebis</t>
         </is>
       </c>
-      <c r="B60" s="16" t="inlineStr">
+      <c r="B61" s="25" t="inlineStr">
         <is>
           <t>Lo aporta Rebis sobre su propia sociedad y su historial</t>
         </is>
       </c>
-      <c r="C60" s="8" t="n">
+      <c r="C61" s="7" t="n">
         <v>825000</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
         <is>
           <t>Gastos de financiación a cargo de Rebis</t>
         </is>
       </c>
-      <c r="B61" s="16" t="inlineStr">
+      <c r="B62" s="17" t="inlineStr">
         <is>
           <t>Rebis retiene el beneficio de la financiación, de modo que no se repercuten al proyecto</t>
         </is>
       </c>
-      <c r="C61" s="17">
-        <f>-C33</f>
+      <c r="C62" s="18">
+        <f>-C34</f>
         <v>-90386.01</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
         <is>
           <t>Aporte neto de Rebis</t>
         </is>
       </c>
-      <c r="B62" s="7" t="n"/>
-      <c r="C62" s="13">
-        <f>C60+C61</f>
+      <c r="B63" s="10" t="n"/>
+      <c r="C63" s="14">
+        <f>C61+C62</f>
         <v>734613.99</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>Aporte de la constructora</t>
         </is>
       </c>
-      <c r="B63" s="16" t="inlineStr">
+      <c r="B64" s="25" t="inlineStr">
         <is>
           <t>Ejecución y financiación de obra</t>
         </is>
       </c>
-      <c r="C63" s="8" t="n">
+      <c r="C64" s="7" t="n">
         <v>325000</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="12" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>Aporte del Inversor</t>
         </is>
       </c>
-      <c r="B64" s="16" t="inlineStr">
+      <c r="B65" s="17" t="inlineStr">
         <is>
           <t>Completa el capital necesario de la actuación</t>
         </is>
       </c>
-      <c r="C64" s="13">
-        <f>C57-C62-C63</f>
+      <c r="C65" s="14">
+        <f>C58-C63-C64</f>
         <v>906254.45</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="18" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t>Total aportes</t>
         </is>
       </c>
-      <c r="B65" s="19" t="n"/>
-      <c r="C65" s="20">
-        <f>C62+C63+C64</f>
+      <c r="B66" s="20" t="n"/>
+      <c r="C66" s="21">
+        <f>C63+C64+C65</f>
         <v>1965868.44</v>
       </c>
     </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="5" t="inlineStr">
+    <row r="68" ht="17" customHeight="1">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>PORCENTAJES DE PARTICIPACIÓN</t>
         </is>
       </c>
-      <c r="B67" s="5" t="n"/>
-      <c r="C67" s="5" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr">
+      <c r="B68" s="4" t="n"/>
+      <c r="C68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
         <is>
           <t>Rebis</t>
         </is>
       </c>
-      <c r="B68" s="7" t="n"/>
-      <c r="C68" s="24">
-        <f>C62/C57*100</f>
+      <c r="B69" s="10" t="n"/>
+      <c r="C69" s="26">
+        <f>C63/C58*100</f>
         <v>37.3684207474</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
         <is>
           <t>Constructora</t>
         </is>
       </c>
-      <c r="B69" s="7" t="n"/>
-      <c r="C69" s="24">
-        <f>C63/C57*100</f>
+      <c r="B70" s="10" t="n"/>
+      <c r="C70" s="26">
+        <f>C64/C58*100</f>
         <v>16.5321337576</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="12" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>Inversor</t>
         </is>
       </c>
-      <c r="B70" s="7" t="n"/>
-      <c r="C70" s="25">
-        <f>C64/C57*100</f>
+      <c r="B71" s="10" t="n"/>
+      <c r="C71" s="27">
+        <f>C65/C58*100</f>
         <v>46.0994454949</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="18" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="19" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B71" s="19" t="n"/>
-      <c r="C71" s="26">
-        <f>C68+C69+C70</f>
+      <c r="B72" s="20" t="n"/>
+      <c r="C72" s="28">
+        <f>C69+C70+C71</f>
         <v>100</v>
       </c>
     </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="5" t="inlineStr">
+    <row r="74" ht="17" customHeight="1">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>RESULTADO DE LA OPERACIÓN</t>
         </is>
       </c>
-      <c r="B73" s="5" t="n"/>
-      <c r="C73" s="5" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="B74" s="4" t="n"/>
+      <c r="C74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>Total costes generales</t>
         </is>
       </c>
-      <c r="B74" s="7" t="n"/>
-      <c r="C74" s="17">
-        <f>$C$7+C22+C33+C41+C46+C50</f>
+      <c r="B75" s="10" t="n"/>
+      <c r="C75" s="18">
+        <f>$C$8+C23+C34+C42+C47+C51</f>
         <v>2165106.91</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="9" t="inlineStr">
         <is>
           <t>Precio de venta estimado</t>
         </is>
       </c>
-      <c r="B75" s="7" t="n"/>
-      <c r="C75" s="17">
-        <f>$C$11</f>
+      <c r="B76" s="10" t="n"/>
+      <c r="C76" s="18">
+        <f>$C$12</f>
         <v>2499200</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>Costes de financiación a cargo de Rebis</t>
         </is>
       </c>
-      <c r="B76" s="16" t="inlineStr">
+      <c r="B77" s="17" t="inlineStr">
         <is>
           <t>Gastos de financiación por adquisición y por venta</t>
         </is>
       </c>
-      <c r="C76" s="17">
-        <f>C33+C50</f>
+      <c r="C77" s="18">
+        <f>C34+C51</f>
         <v>93117.51</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="21" t="inlineStr">
-        <is>
-          <t>Beneficio de la operación  (sin los costes a cargo de Rebis)</t>
-        </is>
-      </c>
-      <c r="B77" s="22" t="n"/>
-      <c r="C77" s="23">
-        <f>$C$11-C74+C76</f>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="22" t="inlineStr">
+        <is>
+          <t>Beneficio de la operación · sin los costes a cargo de Rebis</t>
+        </is>
+      </c>
+      <c r="B78" s="23" t="n"/>
+      <c r="C78" s="24">
+        <f>$C$12-C75+C77</f>
         <v>427210.5999999999</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="6" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>Ganancia de la constructora</t>
         </is>
       </c>
-      <c r="B78" s="16" t="inlineStr">
+      <c r="B79" s="25" t="inlineStr">
         <is>
           <t>Importe fijado por Rebis; única cifra del modelo sin fórmula</t>
         </is>
       </c>
-      <c r="C78" s="8" t="n">
+      <c r="C79" s="7" t="n">
         <v>70846.89999999999</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="6" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t>Honorarios de gestión de Rebis</t>
         </is>
       </c>
-      <c r="B79" s="16" t="inlineStr">
+      <c r="B80" s="17" t="inlineStr">
         <is>
           <t>20 % más IVA sobre el beneficio una vez deducida la constructora</t>
         </is>
       </c>
-      <c r="C79" s="17">
-        <f>ROUND((C77-C78)*0.242,2)</f>
+      <c r="C80" s="18">
+        <f>ROUND((C78-C79)*0.242,2)</f>
         <v>86240.02</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="18" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="19" t="inlineStr">
         <is>
           <t>Beneficio a repartir entre los aportantes</t>
         </is>
       </c>
-      <c r="B80" s="19" t="n"/>
-      <c r="C80" s="20">
-        <f>C77-C78-C79</f>
+      <c r="B81" s="20" t="n"/>
+      <c r="C81" s="21">
+        <f>C78-C79-C80</f>
         <v>270123.6799999998</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="12" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="13" t="inlineStr">
         <is>
           <t>Ganancia del Inversor, antes de impuestos</t>
         </is>
       </c>
-      <c r="B81" s="16" t="inlineStr">
+      <c r="B82" s="17" t="inlineStr">
         <is>
           <t>Su porcentaje de participación sobre el beneficio a repartir</t>
         </is>
       </c>
-      <c r="C81" s="13">
-        <f>ROUND(C80*C70/100,2)</f>
+      <c r="C82" s="14">
+        <f>ROUND(C81*C71/100,2)</f>
         <v>124525.52</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="21" t="inlineStr">
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="22" t="inlineStr">
         <is>
           <t>Rentabilidad del Inversor sobre el capital aportado</t>
         </is>
       </c>
-      <c r="B82" s="22" t="n"/>
-      <c r="C82" s="27">
-        <f>C81/C64*100</f>
+      <c r="B83" s="23" t="n"/>
+      <c r="C83" s="29">
+        <f>C82/C65*100</f>
         <v>13.740679563</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="6" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="9" t="inlineStr">
         <is>
           <t>Rentabilidad antes de los honorarios de Rebis</t>
         </is>
       </c>
-      <c r="B83" s="16" t="inlineStr">
+      <c r="B84" s="17" t="inlineStr">
         <is>
           <t>Equivalencia para comparar con operaciones sin gestión contratada</t>
         </is>
       </c>
-      <c r="C83" s="24">
-        <f>(C81+C79*C70/100)/C64*100</f>
+      <c r="C84" s="26">
+        <f>(C82+C80*C71/100)/C65*100</f>
         <v>18.1275458581</v>
       </c>
     </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="5" t="inlineStr">
+    <row r="86" ht="17" customHeight="1">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
-      <c r="B85" s="5" t="n"/>
-      <c r="C85" s="5" t="n"/>
-    </row>
-    <row r="86" ht="13" customHeight="1">
-      <c r="A86" s="28" t="inlineStr">
-        <is>
-          <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se va liberando mes a mes contra esas cuotas. Figura en el cuadro porque el importe debe estar disponible desde el primer día, pero el coste real de financiación de la operación es la diferencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="13" customHeight="1"/>
-    <row r="88" ht="13" customHeight="1">
-      <c r="A88" s="28" t="inlineStr">
-        <is>
-          <t>2 · Honorarios de Rebis. Se calculan como un 20 % más IVA, equivalente al 24,2 % sobre el beneficio de la operación una vez deducida la ganancia de la constructora. En esta opción Rebis no cobra comisión por la gestión de la hipoteca, porque la toma sobre su propia sociedad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="13" customHeight="1"/>
-    <row r="90" ht="13" customHeight="1">
-      <c r="A90" s="28" t="inlineStr">
-        <is>
-          <t>3 · Rentabilidad. La cifra mostrada es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="13" customHeight="1"/>
-    <row r="92" ht="13" customHeight="1">
-      <c r="A92" s="28" t="inlineStr">
+      <c r="B86" s="4" t="n"/>
+      <c r="C86" s="4" t="n"/>
+    </row>
+    <row r="87" ht="12.5" customHeight="1">
+      <c r="A87" s="30" t="inlineStr">
+        <is>
+          <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes contra esas cuotas. Figura en el cuadro porque el importe debe estar disponible desde el primer día, pero el coste real de financiación de la operación es la diferencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="12.5" customHeight="1"/>
+    <row r="89" ht="12.5" customHeight="1">
+      <c r="A89" s="30" t="inlineStr">
+        <is>
+          <t>2 · Honorarios de Rebis. Un 20 % más IVA, equivalente al 24,2 %, sobre el beneficio de la operación una vez deducida la ganancia de la constructora. Aquí Rebis no cobra comisión por la gestión de la hipoteca, porque la toma sobre su propia sociedad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="12.5" customHeight="1"/>
+    <row r="91" ht="12.5" customHeight="1">
+      <c r="A91" s="30" t="inlineStr">
+        <is>
+          <t>3 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="12.5" customHeight="1"/>
+    <row r="93" ht="12.5" customHeight="1">
+      <c r="A93" s="30" t="inlineStr">
         <is>
           <t>4 · En esta opción el Inversor no figura ante el banco, no presta aval y no constituye ni administra sociedad alguna en España. La financiación bancaria, su coste y su riesgo quedan íntegramente del lado de Rebis, y por eso el apalancamiento no juega a su favor.</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="13" customHeight="1"/>
-    <row r="94" ht="13" customHeight="1">
-      <c r="A94" s="28" t="inlineStr">
-        <is>
-          <t>Las celdas en azul son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="13" customHeight="1"/>
+    <row r="94" ht="12.5" customHeight="1"/>
+    <row r="95" ht="12.5" customHeight="1">
+      <c r="A95" s="30" t="inlineStr">
+        <is>
+          <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="12.5" customHeight="1"/>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="31" t="inlineStr">
+        <is>
+          <t>TRANSFORMAR CON CRITERIO.</t>
+        </is>
+      </c>
+      <c r="B98" s="20" t="n"/>
+      <c r="C98" s="32" t="inlineStr">
+        <is>
+          <t>rebis.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A86:C87"/>
-    <mergeCell ref="A90:C91"/>
-    <mergeCell ref="A94:C95"/>
-    <mergeCell ref="A88:C89"/>
-    <mergeCell ref="A92:C93"/>
+  <mergeCells count="6">
+    <mergeCell ref="A89:C90"/>
+    <mergeCell ref="A91:C92"/>
+    <mergeCell ref="A87:C88"/>
+    <mergeCell ref="A93:C94"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A95:C96"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToWidth="1"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1542,7 +1639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A3:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1550,875 +1647,886 @@
     <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>REBIS · DESARROLLOS INMOBILIARIOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cash-Flow del Inversor  ·  Opción 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Apartamento calle Ruiz Jiménez 3, Madrid  ·  La sociedad titular del inmueble es del Inversor, que toma la hipoteca a su nombre  ·  Escenario conservador</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="1" ht="52" customHeight="1"/>
+    <row r="2" ht="8" customHeight="1"/>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Cash-Flow del Inversor · Opción 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Apartamento calle Ruiz Jiménez 3, Madrid.  La sociedad titular del inmueble es del Inversor, que toma la hipoteca a su nombre.  Escenario conservador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="6" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>RESUMEN DE COMPRA Y VENTA</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Precio de compra</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="8" t="n">
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="n">
         <v>1500000</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>M2 construidos</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="9" t="n">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="8" t="n">
         <v>176</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Precio del m2 de compra</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="10">
-        <f>C7/C8</f>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="11">
+        <f>C8/C9</f>
         <v>8522.7272727273</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Precio del m2 de venta</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="11" t="n">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="12" t="n">
         <v>14200</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Precio de venta estimado</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="13">
-        <f>C10*C8</f>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="14">
+        <f>C11*C9</f>
         <v>2499200</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>COSTES  ·  IMPORTES CON IVA INCLUIDO</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>ACTUACIÓN</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>CONCEPTO</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>IMPORTE</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Adquisición</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Comisión inmobiliaria</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>45375</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="16" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="n"/>
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Honorarios legales por análisis de documentación</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C17" s="18" t="n">
         <v>1270.5</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="16" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="9" t="n"/>
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>ITP · IVA · AJD</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C18" s="18" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="n"/>
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Notaría</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C19" s="18" t="n">
         <v>2700</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="16" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Gestoría</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C20" s="18" t="n">
         <v>494</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="16" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Registro de la propiedad</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C21" s="18" t="n">
         <v>1600</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="n"/>
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>IBI y tasas de basuras, proporcional 2026</t>
         </is>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C22" s="18" t="n">
         <v>875</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Total adquisición</t>
         </is>
       </c>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="20">
-        <f>SUM(C15:C21)</f>
+      <c r="B23" s="20" t="n"/>
+      <c r="C23" s="21">
+        <f>SUM(C16:C22)</f>
         <v>82314.5</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Financiación bancaria</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Tasación</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C24" s="18" t="n">
         <v>605</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="16" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="n"/>
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Pago otorgamiento de hipoteca (AJD)</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C25" s="18" t="n">
         <v>9000</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="16" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="9" t="n"/>
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Comisión por otorgamiento de hipoteca</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C26" s="18" t="n">
         <v>2475</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="16" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="n"/>
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>Contribución especial Fundación CaixaBank</t>
         </is>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C27" s="18" t="n">
         <v>1200</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>Pignoración (fondo recuperable, ver nota 1)</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="n">
+    <row r="28">
+      <c r="A28" s="9" t="n"/>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Pignoración · fondo recuperable, ver nota 1</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="n">
         <v>38000</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="16" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="9" t="n"/>
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Gastos de hipoteca</t>
         </is>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C29" s="18" t="n">
         <v>35062.5</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="16" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="n"/>
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Seguro de responsabilidad civil</t>
         </is>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C30" s="18" t="n">
         <v>649.51</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="16" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="n"/>
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Notaría</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C31" s="18" t="n">
         <v>2000</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="16" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="n"/>
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Gestoría</t>
         </is>
       </c>
-      <c r="C31" s="17" t="n">
+      <c r="C32" s="18" t="n">
         <v>494</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="16" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>Registro de la propiedad</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C33" s="18" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Total financiación bancaria</t>
         </is>
       </c>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="20">
-        <f>SUM(C23:C32)</f>
+      <c r="B34" s="20" t="n"/>
+      <c r="C34" s="21">
+        <f>SUM(C24:C33)</f>
         <v>90386.01</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>Reforma</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>Seguro de incendio</t>
         </is>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C35" s="18" t="n">
         <v>703.9400000000001</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="16" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="9" t="n"/>
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>Asamblea para aprobación de reformas en áreas comunes</t>
         </is>
       </c>
-      <c r="C35" s="17" t="n">
+      <c r="C36" s="18" t="n">
         <v>150</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="16" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>Obra</t>
         </is>
       </c>
-      <c r="C36" s="17" t="n">
+      <c r="C37" s="18" t="n">
         <v>325000</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="16" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="9" t="n"/>
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>Muebles</t>
         </is>
       </c>
-      <c r="C37" s="17" t="n">
+      <c r="C38" s="18" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="16" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Imprevistos</t>
         </is>
       </c>
-      <c r="C38" s="17" t="n">
+      <c r="C39" s="18" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="16" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>Honorarios de interiorismo y arquitectura</t>
         </is>
       </c>
-      <c r="C39" s="17" t="n">
+      <c r="C40" s="18" t="n">
         <v>6500</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="16" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="n"/>
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>Impuestos corrientes durante la ejecución de obra</t>
         </is>
       </c>
-      <c r="C40" s="17" t="n">
+      <c r="C41" s="18" t="n">
         <v>5300</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="18" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>Total reforma</t>
         </is>
       </c>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="20">
-        <f>SUM(C34:C40)</f>
+      <c r="B42" s="20" t="n"/>
+      <c r="C42" s="21">
+        <f>SUM(C35:C41)</f>
         <v>382653.94</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Venta</t>
         </is>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B43" s="17" t="inlineStr">
         <is>
           <t>Fotografía y afines</t>
         </is>
       </c>
-      <c r="C42" s="17" t="n">
+      <c r="C43" s="18" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="16" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="9" t="n"/>
+      <c r="B44" s="17" t="inlineStr">
         <is>
           <t>IBI y tasas de basuras, proporcional 2027</t>
         </is>
       </c>
-      <c r="C43" s="17" t="n">
+      <c r="C44" s="18" t="n">
         <v>400</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="16" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="9" t="n"/>
+      <c r="B45" s="17" t="inlineStr">
         <is>
           <t>Comisión inmobiliaria</t>
         </is>
       </c>
-      <c r="C44" s="17">
-        <f>ROUND($C$11*0.0363,2)</f>
+      <c r="C45" s="18">
+        <f>ROUND($C$12*0.0363,2)</f>
         <v>90720.96</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="16" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="9" t="n"/>
+      <c r="B46" s="17" t="inlineStr">
         <is>
           <t>Plusvalía municipal</t>
         </is>
       </c>
-      <c r="C45" s="17" t="n">
+      <c r="C46" s="18" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="16" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="9" t="n"/>
+      <c r="B47" s="17" t="inlineStr">
         <is>
           <t>Comisión por cancelación de hipoteca</t>
         </is>
       </c>
-      <c r="C46" s="17" t="n">
+      <c r="C47" s="18" t="n">
         <v>1237.5</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="16" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="9" t="n"/>
+      <c r="B48" s="17" t="inlineStr">
         <is>
           <t>Gestoría por cancelación de hipoteca</t>
         </is>
       </c>
-      <c r="C47" s="17" t="n">
+      <c r="C48" s="18" t="n">
         <v>494</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="16" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="9" t="n"/>
+      <c r="B49" s="17" t="inlineStr">
         <is>
           <t>Registro de la propiedad por cancelación</t>
         </is>
       </c>
-      <c r="C48" s="17" t="n">
+      <c r="C49" s="18" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="18" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>Total venta</t>
         </is>
       </c>
-      <c r="B49" s="19" t="n"/>
-      <c r="C49" s="20">
-        <f>SUM(C42:C48)</f>
+      <c r="B50" s="20" t="n"/>
+      <c r="C50" s="21">
+        <f>SUM(C43:C49)</f>
         <v>109752.46</v>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  (SIN GASTOS DE VENTA)</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+    <row r="52" ht="17" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  ·  SIN GASTOS DE VENTA</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>Compra del apartamento</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="17">
-        <f>$C$7</f>
+      <c r="B53" s="10" t="n"/>
+      <c r="C53" s="18">
+        <f>$C$8</f>
         <v>1500000</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>Gastos derivados de la adquisición</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="17">
-        <f>C22</f>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="18">
+        <f>C23</f>
         <v>82314.5</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>Gastos de financiación bancaria</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="17">
-        <f>C33</f>
+      <c r="B55" s="10" t="n"/>
+      <c r="C55" s="18">
+        <f>C34</f>
         <v>90386.01</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Gastos de reforma</t>
         </is>
       </c>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="17">
-        <f>C41</f>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="18">
+        <f>C42</f>
         <v>382653.94</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>Fotografía y afines</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n"/>
-      <c r="C56" s="17" t="n">
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="18" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="21" t="inlineStr">
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Capital necesario</t>
         </is>
       </c>
-      <c r="B57" s="22" t="n"/>
-      <c r="C57" s="23">
-        <f>SUM(C52:C56)</f>
+      <c r="B58" s="23" t="n"/>
+      <c r="C58" s="24">
+        <f>SUM(C53:C57)</f>
         <v>2056254.45</v>
       </c>
     </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="60" ht="17" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>APORTES DE CAPITAL</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n"/>
-      <c r="C59" s="5" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>Aporte bancario</t>
         </is>
       </c>
-      <c r="B60" s="16" t="inlineStr">
+      <c r="B61" s="25" t="inlineStr">
         <is>
           <t>Hipoteca a nombre de la sociedad del Inversor, con su aval personal</t>
         </is>
       </c>
-      <c r="C60" s="8" t="n">
+      <c r="C61" s="7" t="n">
         <v>825000</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>Aporte de la constructora</t>
         </is>
       </c>
-      <c r="B61" s="16" t="inlineStr">
+      <c r="B62" s="25" t="inlineStr">
         <is>
           <t>Ejecución y financiación de obra</t>
         </is>
       </c>
-      <c r="C61" s="8" t="n">
+      <c r="C62" s="7" t="n">
         <v>325000</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
         <is>
           <t>Aporte del Inversor</t>
         </is>
       </c>
-      <c r="B62" s="16" t="inlineStr">
+      <c r="B63" s="17" t="inlineStr">
         <is>
           <t>Completa el capital necesario de la actuación</t>
         </is>
       </c>
-      <c r="C62" s="13">
-        <f>C57-C60-C61</f>
+      <c r="C63" s="14">
+        <f>C58-C61-C62</f>
         <v>906254.45</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="18" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="19" t="inlineStr">
         <is>
           <t>Total aportes</t>
         </is>
       </c>
-      <c r="B63" s="19" t="n"/>
-      <c r="C63" s="20">
-        <f>SUM(C60:C62)</f>
+      <c r="B64" s="20" t="n"/>
+      <c r="C64" s="21">
+        <f>SUM(C61:C63)</f>
         <v>2056254.45</v>
       </c>
     </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="5" t="inlineStr">
+    <row r="66" ht="17" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>RESULTADO DE LA OPERACIÓN</t>
         </is>
       </c>
-      <c r="B65" s="5" t="n"/>
-      <c r="C65" s="5" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="B66" s="4" t="n"/>
+      <c r="C66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="inlineStr">
         <is>
           <t>Total costes</t>
         </is>
       </c>
-      <c r="B66" s="16" t="inlineStr">
-        <is>
-          <t>Sin el gasto de pignoración, que es un fondo recuperable (ver nota 1)</t>
-        </is>
-      </c>
-      <c r="C66" s="17">
-        <f>$C$7+C22+C33+C41+C49-38000</f>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>Sin el gasto de pignoración, que es un fondo recuperable · ver nota 1</t>
+        </is>
+      </c>
+      <c r="C67" s="18">
+        <f>$C$8+C23+C34+C42+C50-38000</f>
         <v>2127106.91</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
         <is>
           <t>Precio de venta estimado</t>
         </is>
       </c>
-      <c r="B67" s="7" t="n"/>
-      <c r="C67" s="17">
-        <f>$C$11</f>
+      <c r="B68" s="10" t="n"/>
+      <c r="C68" s="18">
+        <f>$C$12</f>
         <v>2499200</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="21" t="inlineStr">
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>Beneficio de la operación</t>
         </is>
       </c>
-      <c r="B68" s="22" t="n"/>
-      <c r="C68" s="23">
-        <f>$C$11-C66</f>
+      <c r="B69" s="23" t="n"/>
+      <c r="C69" s="24">
+        <f>$C$12-C67</f>
         <v>372093.0899999999</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>Ganancia de la constructora</t>
         </is>
       </c>
-      <c r="B69" s="16" t="inlineStr">
+      <c r="B70" s="25" t="inlineStr">
         <is>
           <t>Importe fijado por Rebis; única cifra del modelo sin fórmula</t>
         </is>
       </c>
-      <c r="C69" s="8" t="n">
+      <c r="C70" s="7" t="n">
         <v>71924.83</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
         <is>
           <t>Honorarios de gestión de Rebis</t>
         </is>
       </c>
-      <c r="B70" s="16" t="inlineStr">
+      <c r="B71" s="17" t="inlineStr">
         <is>
           <t>20 % más IVA sobre el beneficio una vez deducida la constructora</t>
         </is>
       </c>
-      <c r="C70" s="17">
-        <f>ROUND((C68-C69)*0.242,2)</f>
+      <c r="C71" s="18">
+        <f>ROUND((C69-C70)*0.242,2)</f>
         <v>72640.72</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
         <is>
           <t>Honorarios de Rebis por gestión y tramitación de la hipoteca</t>
         </is>
       </c>
-      <c r="B71" s="16" t="inlineStr">
+      <c r="B72" s="17" t="inlineStr">
         <is>
           <t>2 % más IVA sobre el importe de hipoteca concedido</t>
         </is>
       </c>
-      <c r="C71" s="17">
-        <f>ROUND(C60*0.02*1.21,2)</f>
+      <c r="C72" s="18">
+        <f>ROUND(C61*0.02*1.21,2)</f>
         <v>19965</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
         <is>
           <t>Ganancia del Inversor, antes de impuestos</t>
         </is>
       </c>
-      <c r="B72" s="16" t="inlineStr">
+      <c r="B73" s="17" t="inlineStr">
         <is>
           <t>Recibe la totalidad del resultado restante</t>
         </is>
       </c>
-      <c r="C72" s="13">
-        <f>C68-C69-C70-C71</f>
+      <c r="C73" s="14">
+        <f>C69-C70-C71-C72</f>
         <v>207562.5399999998</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="21" t="inlineStr">
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="22" t="inlineStr">
         <is>
           <t>Rentabilidad del Inversor sobre el capital aportado</t>
         </is>
       </c>
-      <c r="B73" s="22" t="n"/>
-      <c r="C73" s="27">
-        <f>C72/C62*100</f>
+      <c r="B74" s="23" t="n"/>
+      <c r="C74" s="29">
+        <f>C73/C63*100</f>
         <v>22.9033402264</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>Rentabilidad antes de los honorarios de Rebis</t>
         </is>
       </c>
-      <c r="B74" s="16" t="inlineStr">
+      <c r="B75" s="17" t="inlineStr">
         <is>
           <t>Equivalencia para comparar con operaciones sin gestión contratada</t>
         </is>
       </c>
-      <c r="C74" s="24">
-        <f>(C72+C70+C71)/C62*100</f>
+      <c r="C75" s="26">
+        <f>(C73+C71+C72)/C63*100</f>
         <v>33.1218522568</v>
       </c>
     </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="5" t="inlineStr">
+    <row r="77" ht="17" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
-      <c r="B76" s="5" t="n"/>
-      <c r="C76" s="5" t="n"/>
-    </row>
-    <row r="77" ht="13" customHeight="1">
-      <c r="A77" s="28" t="inlineStr">
-        <is>
-          <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se va liberando mes a mes y vuelve al Inversor, de modo que en esta opción no se computa como coste de la operación, aunque el importe debe estar disponible desde el primer día.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="13" customHeight="1"/>
-    <row r="79" ht="13" customHeight="1">
-      <c r="A79" s="28" t="inlineStr">
-        <is>
-          <t>2 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio una vez deducida la ganancia de la constructora, más un 2 % más IVA sobre el importe de hipoteca efectivamente concedido, en contraprestación por la gestión de la financiación y por el aval que Rebis aporta ante el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="13" customHeight="1"/>
-    <row r="81" ht="13" customHeight="1">
-      <c r="A81" s="28" t="inlineStr">
-        <is>
-          <t>3 · Rentabilidad. La cifra mostrada es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="13" customHeight="1"/>
-    <row r="83" ht="13" customHeight="1">
-      <c r="A83" s="28" t="inlineStr">
+      <c r="B77" s="4" t="n"/>
+      <c r="C77" s="4" t="n"/>
+    </row>
+    <row r="78" ht="12.5" customHeight="1">
+      <c r="A78" s="30" t="inlineStr">
+        <is>
+          <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes y vuelve al Inversor, de modo que aquí no se computa como coste de la operación, aunque el importe debe estar disponible desde el primer día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="12.5" customHeight="1"/>
+    <row r="80" ht="12.5" customHeight="1">
+      <c r="A80" s="30" t="inlineStr">
+        <is>
+          <t>2 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio una vez deducida la ganancia de la constructora, más un 2 % más IVA sobre el importe de hipoteca efectivamente concedido, por la gestión de la financiación y por el aval que Rebis aporta ante el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="12.5" customHeight="1"/>
+    <row r="82" ht="12.5" customHeight="1">
+      <c r="A82" s="30" t="inlineStr">
+        <is>
+          <t>3 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="12.5" customHeight="1"/>
+    <row r="84" ht="12.5" customHeight="1">
+      <c r="A84" s="30" t="inlineStr">
         <is>
           <t>4 · En esta opción el Inversor constituye y administra la sociedad española, toma la hipoteca a su nombre y presta aval personal con su patrimonio. A cambio, el apalancamiento juega a su favor y recibe la totalidad del resultado restante, no una participación sobre él.</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="13" customHeight="1"/>
-    <row r="85" ht="13" customHeight="1">
-      <c r="A85" s="28" t="inlineStr">
-        <is>
-          <t>Las celdas en azul son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="13" customHeight="1"/>
+    <row r="85" ht="12.5" customHeight="1"/>
+    <row r="86" ht="12.5" customHeight="1">
+      <c r="A86" s="30" t="inlineStr">
+        <is>
+          <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="12.5" customHeight="1"/>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="31" t="inlineStr">
+        <is>
+          <t>TRANSFORMAR CON CRITERIO.</t>
+        </is>
+      </c>
+      <c r="B89" s="20" t="n"/>
+      <c r="C89" s="32" t="inlineStr">
+        <is>
+          <t>rebis.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A77:C78"/>
-    <mergeCell ref="A85:C86"/>
-    <mergeCell ref="A79:C80"/>
-    <mergeCell ref="A83:C84"/>
-    <mergeCell ref="A81:C82"/>
+  <mergeCells count="6">
+    <mergeCell ref="A86:C87"/>
+    <mergeCell ref="A82:C83"/>
+    <mergeCell ref="A80:C81"/>
+    <mergeCell ref="A84:C85"/>
+    <mergeCell ref="A78:C79"/>
+    <mergeCell ref="A4:C4"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToWidth="1"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corregir el libro para que Google pueda leer su texto
El openpyxl de este entorno escribe todas las cadenas como inlineStr y no
genera xl/sharedStrings.xml: 99 cadenas en línea solo en la primera hoja. Es
OOXML válido, pero el importador de Google no lo interpreta y el libro se abre
sin texto alguno, que es lo que estaba pasando al abrirlo desde Drive.

tabla_cadenas.py reescribe el paquete con la tabla de cadenas compartidas —108
entradas, cero en línea— y registra la parte en [Content_Types].xml y en las
relaciones del libro. Las fórmulas, los valores cacheados y el logotipo quedan
intactos y las cifras no se mueven.

Las dos opciones quedan además como Hojas de cálculo nativas en la carpeta de
Drive, cargadas como TSV con locale español, porque el conector corrompe las
subidas binarias.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3Mnw54UTuPQAtnGvXf7kT
</commit_message>
<xml_diff>
--- a/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
+++ b/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
@@ -13,6 +13,335 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="108">
+  <si>
+    <t>Cash-Flow del Inversor · Opción 1</t>
+  </si>
+  <si>
+    <t>Apartamento calle Ruiz Jiménez 3, Madrid.  La operación se canaliza a través de la sociedad de Rebis y el Inversor entra mediante préstamo participativo.  Escenario conservador.</t>
+  </si>
+  <si>
+    <t>RESUMEN DE COMPRA Y VENTA</t>
+  </si>
+  <si>
+    <t>Precio de compra</t>
+  </si>
+  <si>
+    <t>M2 construidos</t>
+  </si>
+  <si>
+    <t>Precio del m2 de compra</t>
+  </si>
+  <si>
+    <t>Precio del m2 de venta</t>
+  </si>
+  <si>
+    <t>Precio de venta estimado</t>
+  </si>
+  <si>
+    <t>COSTES  ·  IMPORTES CON IVA INCLUIDO</t>
+  </si>
+  <si>
+    <t>ACTUACIÓN</t>
+  </si>
+  <si>
+    <t>CONCEPTO</t>
+  </si>
+  <si>
+    <t>IMPORTE</t>
+  </si>
+  <si>
+    <t>Adquisición</t>
+  </si>
+  <si>
+    <t>Comisión inmobiliaria</t>
+  </si>
+  <si>
+    <t>Honorarios legales por análisis de documentación</t>
+  </si>
+  <si>
+    <t>ITP · IVA · AJD</t>
+  </si>
+  <si>
+    <t>Notaría</t>
+  </si>
+  <si>
+    <t>Gestoría</t>
+  </si>
+  <si>
+    <t>Registro de la propiedad</t>
+  </si>
+  <si>
+    <t>IBI y tasas de basuras, proporcional 2026</t>
+  </si>
+  <si>
+    <t>Total adquisición</t>
+  </si>
+  <si>
+    <t>Financiación bancaria</t>
+  </si>
+  <si>
+    <t>Tasación</t>
+  </si>
+  <si>
+    <t>Pago otorgamiento de hipoteca (AJD)</t>
+  </si>
+  <si>
+    <t>Comisión por otorgamiento de hipoteca</t>
+  </si>
+  <si>
+    <t>Contribución especial Fundación CaixaBank</t>
+  </si>
+  <si>
+    <t>Pignoración · fondo recuperable, ver nota 1</t>
+  </si>
+  <si>
+    <t>Gastos de hipoteca</t>
+  </si>
+  <si>
+    <t>Seguro de responsabilidad civil</t>
+  </si>
+  <si>
+    <t>Total financiación bancaria</t>
+  </si>
+  <si>
+    <t>Reforma</t>
+  </si>
+  <si>
+    <t>Seguro de incendio</t>
+  </si>
+  <si>
+    <t>Asamblea para aprobación de reformas en áreas comunes</t>
+  </si>
+  <si>
+    <t>Obra</t>
+  </si>
+  <si>
+    <t>Muebles</t>
+  </si>
+  <si>
+    <t>Imprevistos</t>
+  </si>
+  <si>
+    <t>Honorarios de interiorismo y arquitectura</t>
+  </si>
+  <si>
+    <t>Impuestos corrientes durante la ejecución de obra</t>
+  </si>
+  <si>
+    <t>Total reforma</t>
+  </si>
+  <si>
+    <t>Venta</t>
+  </si>
+  <si>
+    <t>Fotografía y afines</t>
+  </si>
+  <si>
+    <t>IBI y tasas de basuras, proporcional 2027</t>
+  </si>
+  <si>
+    <t>Plusvalía municipal</t>
+  </si>
+  <si>
+    <t>Total venta</t>
+  </si>
+  <si>
+    <t>Financiación por venta</t>
+  </si>
+  <si>
+    <t>Comisión por cancelación de hipoteca</t>
+  </si>
+  <si>
+    <t>Gestoría por cancelación de hipoteca</t>
+  </si>
+  <si>
+    <t>Registro de la propiedad por cancelación</t>
+  </si>
+  <si>
+    <t>Total financiación por venta</t>
+  </si>
+  <si>
+    <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  ·  SIN GASTOS DE VENTA NI DE FINANCIACIÓN</t>
+  </si>
+  <si>
+    <t>Compra del apartamento</t>
+  </si>
+  <si>
+    <t>Gastos derivados de la adquisición</t>
+  </si>
+  <si>
+    <t>Gastos de reforma</t>
+  </si>
+  <si>
+    <t>Capital necesario</t>
+  </si>
+  <si>
+    <t>APORTES DE CAPITAL</t>
+  </si>
+  <si>
+    <t>Aporte de capital bancario · Rebis</t>
+  </si>
+  <si>
+    <t>Lo aporta Rebis sobre su propia sociedad y su historial</t>
+  </si>
+  <si>
+    <t>Gastos de financiación a cargo de Rebis</t>
+  </si>
+  <si>
+    <t>Rebis retiene el beneficio de la financiación, de modo que no se repercuten al proyecto</t>
+  </si>
+  <si>
+    <t>Aporte neto de Rebis</t>
+  </si>
+  <si>
+    <t>Aporte de la constructora</t>
+  </si>
+  <si>
+    <t>Ejecución y financiación de obra</t>
+  </si>
+  <si>
+    <t>Aporte del Inversor</t>
+  </si>
+  <si>
+    <t>Completa el capital necesario de la actuación</t>
+  </si>
+  <si>
+    <t>Total aportes</t>
+  </si>
+  <si>
+    <t>PORCENTAJES DE PARTICIPACIÓN</t>
+  </si>
+  <si>
+    <t>Rebis</t>
+  </si>
+  <si>
+    <t>Constructora</t>
+  </si>
+  <si>
+    <t>Inversor</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>RESULTADO DE LA OPERACIÓN</t>
+  </si>
+  <si>
+    <t>Total costes generales</t>
+  </si>
+  <si>
+    <t>Costes de financiación a cargo de Rebis</t>
+  </si>
+  <si>
+    <t>Gastos de financiación por adquisición y por venta</t>
+  </si>
+  <si>
+    <t>Beneficio de la operación · sin los costes a cargo de Rebis</t>
+  </si>
+  <si>
+    <t>Ganancia de la constructora</t>
+  </si>
+  <si>
+    <t>Importe fijado por Rebis; única cifra del modelo sin fórmula</t>
+  </si>
+  <si>
+    <t>Honorarios de gestión de Rebis</t>
+  </si>
+  <si>
+    <t>20 % más IVA sobre el beneficio una vez deducida la constructora</t>
+  </si>
+  <si>
+    <t>Beneficio a repartir entre los aportantes</t>
+  </si>
+  <si>
+    <t>Ganancia del Inversor, antes de impuestos</t>
+  </si>
+  <si>
+    <t>Su porcentaje de participación sobre el beneficio a repartir</t>
+  </si>
+  <si>
+    <t>Rentabilidad del Inversor sobre el capital aportado</t>
+  </si>
+  <si>
+    <t>Rentabilidad antes de los honorarios de Rebis</t>
+  </si>
+  <si>
+    <t>Equivalencia para comparar con operaciones sin gestión contratada</t>
+  </si>
+  <si>
+    <t>NOTAS</t>
+  </si>
+  <si>
+    <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes contra esas cuotas. Figura en el cuadro porque el importe debe estar disponible desde el primer día, pero el coste real de financiación de la operación es la diferencia.</t>
+  </si>
+  <si>
+    <t>2 · Honorarios de Rebis. Un 20 % más IVA, equivalente al 24,2 %, sobre el beneficio de la operación una vez deducida la ganancia de la constructora. Aquí Rebis no cobra comisión por la gestión de la hipoteca, porque la toma sobre su propia sociedad.</t>
+  </si>
+  <si>
+    <t>3 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
+  </si>
+  <si>
+    <t>4 · En esta opción el Inversor no figura ante el banco, no presta aval y no constituye ni administra sociedad alguna en España. La financiación bancaria, su coste y su riesgo quedan íntegramente del lado de Rebis, y por eso el apalancamiento no juega a su favor.</t>
+  </si>
+  <si>
+    <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
+  </si>
+  <si>
+    <t>TRANSFORMAR CON CRITERIO.</t>
+  </si>
+  <si>
+    <t>rebis.com</t>
+  </si>
+  <si>
+    <t>Cash-Flow del Inversor · Opción 2</t>
+  </si>
+  <si>
+    <t>Apartamento calle Ruiz Jiménez 3, Madrid.  La sociedad titular del inmueble es del Inversor, que toma la hipoteca a su nombre.  Escenario conservador.</t>
+  </si>
+  <si>
+    <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  ·  SIN GASTOS DE VENTA</t>
+  </si>
+  <si>
+    <t>Gastos de financiación bancaria</t>
+  </si>
+  <si>
+    <t>Aporte bancario</t>
+  </si>
+  <si>
+    <t>Hipoteca a nombre de la sociedad del Inversor, con su aval personal</t>
+  </si>
+  <si>
+    <t>Total costes</t>
+  </si>
+  <si>
+    <t>Sin el gasto de pignoración, que es un fondo recuperable · ver nota 1</t>
+  </si>
+  <si>
+    <t>Beneficio de la operación</t>
+  </si>
+  <si>
+    <t>Honorarios de Rebis por gestión y tramitación de la hipoteca</t>
+  </si>
+  <si>
+    <t>2 % más IVA sobre el importe de hipoteca concedido</t>
+  </si>
+  <si>
+    <t>Recibe la totalidad del resultado restante</t>
+  </si>
+  <si>
+    <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes y vuelve al Inversor, de modo que aquí no se computa como coste de la operación, aunque el importe debe estar disponible desde el primer día.</t>
+  </si>
+  <si>
+    <t>2 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio una vez deducida la ganancia de la constructora, más un 2 % más IVA sobre el importe de hipoteca efectivamente concedido, por la gestión de la financiación y por el aval que Rebis aporta ante el banco.</t>
+  </si>
+  <si>
+    <t>4 · En esta opción el Inversor constituye y administra la sociedad española, toma la hipoteca a su nombre y presta aval personal con su patrimonio. A cambio, el apalancamiento juega a su favor y recibe la totalidad del resultado restante, no una participación sobre él.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -655,17 +984,13 @@
     <row r="1" ht="52" customHeight="1"/>
     <row r="2" ht="8" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Cash-Flow del Inversor · Opción 1</t>
-        </is>
+      <c r="A3" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Apartamento calle Ruiz Jiménez 3, Madrid.  La operación se canaliza a través de la sociedad de Rebis y el Inversor entra mediante préstamo participativo.  Escenario conservador.</t>
-        </is>
+      <c r="A4" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="6" customHeight="1">
@@ -674,19 +999,15 @@
       <c r="C5" s="3" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>RESUMEN DE COMPRA Y VENTA</t>
-        </is>
+      <c r="A7" s="4" t="s">
+        <v>2</v>
       </c>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Precio de compra</t>
-        </is>
+      <c r="A8" s="5" t="s">
+        <v>3</v>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="n">
@@ -694,10 +1015,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>M2 construidos</t>
-        </is>
+      <c r="A9" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="8" t="n">
@@ -705,10 +1024,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Precio del m2 de compra</t>
-        </is>
+      <c r="A10" s="9" t="s">
+        <v>5</v>
       </c>
       <c r="B10" s="10" t="n"/>
       <c r="C10" s="11">
@@ -717,10 +1034,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Precio del m2 de venta</t>
-        </is>
+      <c r="A11" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="12" t="n">
@@ -728,10 +1043,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Precio de venta estimado</t>
-        </is>
+      <c r="A12" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="14">
@@ -740,41 +1053,29 @@
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>COSTES  ·  IMPORTES CON IVA INCLUIDO</t>
-        </is>
+      <c r="A14" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="B14" s="4" t="n"/>
       <c r="C14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>ACTUACIÓN</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>CONCEPTO</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>IMPORTE</t>
-        </is>
+      <c r="A15" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Adquisición</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>Comisión inmobiliaria</t>
-        </is>
+      <c r="A16" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>13</v>
       </c>
       <c r="C16" s="18" t="n">
         <v>45375</v>
@@ -782,10 +1083,8 @@
     </row>
     <row r="17">
       <c r="A17" s="9" t="n"/>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Honorarios legales por análisis de documentación</t>
-        </is>
+      <c r="B17" s="17" t="s">
+        <v>14</v>
       </c>
       <c r="C17" s="18" t="n">
         <v>1270.5</v>
@@ -793,10 +1092,8 @@
     </row>
     <row r="18">
       <c r="A18" s="9" t="n"/>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>ITP · IVA · AJD</t>
-        </is>
+      <c r="B18" s="17" t="s">
+        <v>15</v>
       </c>
       <c r="C18" s="18" t="n">
         <v>30000</v>
@@ -804,10 +1101,8 @@
     </row>
     <row r="19">
       <c r="A19" s="9" t="n"/>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>Notaría</t>
-        </is>
+      <c r="B19" s="17" t="s">
+        <v>16</v>
       </c>
       <c r="C19" s="18" t="n">
         <v>2700</v>
@@ -815,10 +1110,8 @@
     </row>
     <row r="20">
       <c r="A20" s="9" t="n"/>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Gestoría</t>
-        </is>
+      <c r="B20" s="17" t="s">
+        <v>17</v>
       </c>
       <c r="C20" s="18" t="n">
         <v>494</v>
@@ -826,10 +1119,8 @@
     </row>
     <row r="21">
       <c r="A21" s="9" t="n"/>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Registro de la propiedad</t>
-        </is>
+      <c r="B21" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="C21" s="18" t="n">
         <v>1600</v>
@@ -837,20 +1128,16 @@
     </row>
     <row r="22">
       <c r="A22" s="9" t="n"/>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>IBI y tasas de basuras, proporcional 2026</t>
-        </is>
+      <c r="B22" s="17" t="s">
+        <v>19</v>
       </c>
       <c r="C22" s="18" t="n">
         <v>875</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>Total adquisición</t>
-        </is>
+      <c r="A23" s="19" t="s">
+        <v>20</v>
       </c>
       <c r="B23" s="20" t="n"/>
       <c r="C23" s="21">
@@ -859,15 +1146,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Financiación bancaria</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>Tasación</t>
-        </is>
+      <c r="A24" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>22</v>
       </c>
       <c r="C24" s="18" t="n">
         <v>605</v>
@@ -875,10 +1158,8 @@
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Pago otorgamiento de hipoteca (AJD)</t>
-        </is>
+      <c r="B25" s="17" t="s">
+        <v>23</v>
       </c>
       <c r="C25" s="18" t="n">
         <v>9000</v>
@@ -886,10 +1167,8 @@
     </row>
     <row r="26">
       <c r="A26" s="9" t="n"/>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>Comisión por otorgamiento de hipoteca</t>
-        </is>
+      <c r="B26" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="C26" s="18" t="n">
         <v>2475</v>
@@ -897,10 +1176,8 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>Contribución especial Fundación CaixaBank</t>
-        </is>
+      <c r="B27" s="17" t="s">
+        <v>25</v>
       </c>
       <c r="C27" s="18" t="n">
         <v>1200</v>
@@ -908,10 +1185,8 @@
     </row>
     <row r="28">
       <c r="A28" s="9" t="n"/>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>Pignoración · fondo recuperable, ver nota 1</t>
-        </is>
+      <c r="B28" s="17" t="s">
+        <v>26</v>
       </c>
       <c r="C28" s="18" t="n">
         <v>38000</v>
@@ -919,10 +1194,8 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>Gastos de hipoteca</t>
-        </is>
+      <c r="B29" s="17" t="s">
+        <v>27</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>35062.5</v>
@@ -930,10 +1203,8 @@
     </row>
     <row r="30">
       <c r="A30" s="9" t="n"/>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>Seguro de responsabilidad civil</t>
-        </is>
+      <c r="B30" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="C30" s="18" t="n">
         <v>649.51</v>
@@ -941,10 +1212,8 @@
     </row>
     <row r="31">
       <c r="A31" s="9" t="n"/>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>Notaría</t>
-        </is>
+      <c r="B31" s="17" t="s">
+        <v>16</v>
       </c>
       <c r="C31" s="18" t="n">
         <v>2000</v>
@@ -952,10 +1221,8 @@
     </row>
     <row r="32">
       <c r="A32" s="9" t="n"/>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>Gestoría</t>
-        </is>
+      <c r="B32" s="17" t="s">
+        <v>17</v>
       </c>
       <c r="C32" s="18" t="n">
         <v>494</v>
@@ -963,20 +1230,16 @@
     </row>
     <row r="33">
       <c r="A33" s="9" t="n"/>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>Registro de la propiedad</t>
-        </is>
+      <c r="B33" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="C33" s="18" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>Total financiación bancaria</t>
-        </is>
+      <c r="A34" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B34" s="20" t="n"/>
       <c r="C34" s="21">
@@ -985,15 +1248,11 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>Reforma</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>Seguro de incendio</t>
-        </is>
+      <c r="A35" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>31</v>
       </c>
       <c r="C35" s="18" t="n">
         <v>703.9400000000001</v>
@@ -1001,10 +1260,8 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="n"/>
-      <c r="B36" s="17" t="inlineStr">
-        <is>
-          <t>Asamblea para aprobación de reformas en áreas comunes</t>
-        </is>
+      <c r="B36" s="17" t="s">
+        <v>32</v>
       </c>
       <c r="C36" s="18" t="n">
         <v>150</v>
@@ -1012,10 +1269,8 @@
     </row>
     <row r="37">
       <c r="A37" s="9" t="n"/>
-      <c r="B37" s="17" t="inlineStr">
-        <is>
-          <t>Obra</t>
-        </is>
+      <c r="B37" s="17" t="s">
+        <v>33</v>
       </c>
       <c r="C37" s="18" t="n">
         <v>325000</v>
@@ -1023,10 +1278,8 @@
     </row>
     <row r="38">
       <c r="A38" s="9" t="n"/>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>Muebles</t>
-        </is>
+      <c r="B38" s="17" t="s">
+        <v>34</v>
       </c>
       <c r="C38" s="18" t="n">
         <v>30000</v>
@@ -1034,10 +1287,8 @@
     </row>
     <row r="39">
       <c r="A39" s="9" t="n"/>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>Imprevistos</t>
-        </is>
+      <c r="B39" s="17" t="s">
+        <v>35</v>
       </c>
       <c r="C39" s="18" t="n">
         <v>15000</v>
@@ -1045,10 +1296,8 @@
     </row>
     <row r="40">
       <c r="A40" s="9" t="n"/>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>Honorarios de interiorismo y arquitectura</t>
-        </is>
+      <c r="B40" s="17" t="s">
+        <v>36</v>
       </c>
       <c r="C40" s="18" t="n">
         <v>6500</v>
@@ -1056,20 +1305,16 @@
     </row>
     <row r="41">
       <c r="A41" s="9" t="n"/>
-      <c r="B41" s="17" t="inlineStr">
-        <is>
-          <t>Impuestos corrientes durante la ejecución de obra</t>
-        </is>
+      <c r="B41" s="17" t="s">
+        <v>37</v>
       </c>
       <c r="C41" s="18" t="n">
         <v>5300</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="inlineStr">
-        <is>
-          <t>Total reforma</t>
-        </is>
+      <c r="A42" s="19" t="s">
+        <v>38</v>
       </c>
       <c r="B42" s="20" t="n"/>
       <c r="C42" s="21">
@@ -1078,15 +1323,11 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="B43" s="17" t="inlineStr">
-        <is>
-          <t>Fotografía y afines</t>
-        </is>
+      <c r="A43" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>40</v>
       </c>
       <c r="C43" s="18" t="n">
         <v>900</v>
@@ -1094,10 +1335,8 @@
     </row>
     <row r="44">
       <c r="A44" s="9" t="n"/>
-      <c r="B44" s="17" t="inlineStr">
-        <is>
-          <t>IBI y tasas de basuras, proporcional 2027</t>
-        </is>
+      <c r="B44" s="17" t="s">
+        <v>41</v>
       </c>
       <c r="C44" s="18" t="n">
         <v>400</v>
@@ -1105,10 +1344,8 @@
     </row>
     <row r="45">
       <c r="A45" s="9" t="n"/>
-      <c r="B45" s="17" t="inlineStr">
-        <is>
-          <t>Comisión inmobiliaria</t>
-        </is>
+      <c r="B45" s="17" t="s">
+        <v>13</v>
       </c>
       <c r="C45" s="18">
         <f>ROUND($C$12*0.0363,2)</f>
@@ -1117,20 +1354,16 @@
     </row>
     <row r="46">
       <c r="A46" s="9" t="n"/>
-      <c r="B46" s="17" t="inlineStr">
-        <is>
-          <t>Plusvalía municipal</t>
-        </is>
+      <c r="B46" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="C46" s="18" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="inlineStr">
-        <is>
-          <t>Total venta</t>
-        </is>
+      <c r="A47" s="19" t="s">
+        <v>43</v>
       </c>
       <c r="B47" s="20" t="n"/>
       <c r="C47" s="21">
@@ -1139,15 +1372,11 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>Financiación por venta</t>
-        </is>
-      </c>
-      <c r="B48" s="17" t="inlineStr">
-        <is>
-          <t>Comisión por cancelación de hipoteca</t>
-        </is>
+      <c r="A48" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>45</v>
       </c>
       <c r="C48" s="18" t="n">
         <v>1237.5</v>
@@ -1155,10 +1384,8 @@
     </row>
     <row r="49">
       <c r="A49" s="9" t="n"/>
-      <c r="B49" s="17" t="inlineStr">
-        <is>
-          <t>Gestoría por cancelación de hipoteca</t>
-        </is>
+      <c r="B49" s="17" t="s">
+        <v>46</v>
       </c>
       <c r="C49" s="18" t="n">
         <v>494</v>
@@ -1166,20 +1393,16 @@
     </row>
     <row r="50">
       <c r="A50" s="9" t="n"/>
-      <c r="B50" s="17" t="inlineStr">
-        <is>
-          <t>Registro de la propiedad por cancelación</t>
-        </is>
+      <c r="B50" s="17" t="s">
+        <v>47</v>
       </c>
       <c r="C50" s="18" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="19" t="inlineStr">
-        <is>
-          <t>Total financiación por venta</t>
-        </is>
+      <c r="A51" s="19" t="s">
+        <v>48</v>
       </c>
       <c r="B51" s="20" t="n"/>
       <c r="C51" s="21">
@@ -1188,19 +1411,15 @@
       </c>
     </row>
     <row r="53" ht="17" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  ·  SIN GASTOS DE VENTA NI DE FINANCIACIÓN</t>
-        </is>
+      <c r="A53" s="4" t="s">
+        <v>49</v>
       </c>
       <c r="B53" s="4" t="n"/>
       <c r="C53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>Compra del apartamento</t>
-        </is>
+      <c r="A54" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="B54" s="10" t="n"/>
       <c r="C54" s="18">
@@ -1209,10 +1428,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
-        <is>
-          <t>Gastos derivados de la adquisición</t>
-        </is>
+      <c r="A55" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="B55" s="10" t="n"/>
       <c r="C55" s="18">
@@ -1221,10 +1438,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>Gastos de reforma</t>
-        </is>
+      <c r="A56" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="B56" s="10" t="n"/>
       <c r="C56" s="18">
@@ -1233,10 +1448,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="9" t="inlineStr">
-        <is>
-          <t>Fotografía y afines</t>
-        </is>
+      <c r="A57" s="9" t="s">
+        <v>40</v>
       </c>
       <c r="B57" s="10" t="n"/>
       <c r="C57" s="18" t="n">
@@ -1244,10 +1457,8 @@
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
-        <is>
-          <t>Capital necesario</t>
-        </is>
+      <c r="A58" s="22" t="s">
+        <v>53</v>
       </c>
       <c r="B58" s="23" t="n"/>
       <c r="C58" s="24">
@@ -1256,39 +1467,29 @@
       </c>
     </row>
     <row r="60" ht="17" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>APORTES DE CAPITAL</t>
-        </is>
+      <c r="A60" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="B60" s="4" t="n"/>
       <c r="C60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Aporte de capital bancario · Rebis</t>
-        </is>
-      </c>
-      <c r="B61" s="25" t="inlineStr">
-        <is>
-          <t>Lo aporta Rebis sobre su propia sociedad y su historial</t>
-        </is>
+      <c r="A61" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B61" s="25" t="s">
+        <v>56</v>
       </c>
       <c r="C61" s="7" t="n">
         <v>825000</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>Gastos de financiación a cargo de Rebis</t>
-        </is>
-      </c>
-      <c r="B62" s="17" t="inlineStr">
-        <is>
-          <t>Rebis retiene el beneficio de la financiación, de modo que no se repercuten al proyecto</t>
-        </is>
+      <c r="A62" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B62" s="17" t="s">
+        <v>58</v>
       </c>
       <c r="C62" s="18">
         <f>-C34</f>
@@ -1296,10 +1497,8 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>Aporte neto de Rebis</t>
-        </is>
+      <c r="A63" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="B63" s="10" t="n"/>
       <c r="C63" s="14">
@@ -1308,30 +1507,22 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>Aporte de la constructora</t>
-        </is>
-      </c>
-      <c r="B64" s="25" t="inlineStr">
-        <is>
-          <t>Ejecución y financiación de obra</t>
-        </is>
+      <c r="A64" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64" s="25" t="s">
+        <v>61</v>
       </c>
       <c r="C64" s="7" t="n">
         <v>325000</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>Aporte del Inversor</t>
-        </is>
-      </c>
-      <c r="B65" s="17" t="inlineStr">
-        <is>
-          <t>Completa el capital necesario de la actuación</t>
-        </is>
+      <c r="A65" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B65" s="17" t="s">
+        <v>63</v>
       </c>
       <c r="C65" s="14">
         <f>C58-C63-C64</f>
@@ -1339,10 +1530,8 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="19" t="inlineStr">
-        <is>
-          <t>Total aportes</t>
-        </is>
+      <c r="A66" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="B66" s="20" t="n"/>
       <c r="C66" s="21">
@@ -1351,19 +1540,15 @@
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>PORCENTAJES DE PARTICIPACIÓN</t>
-        </is>
+      <c r="A68" s="4" t="s">
+        <v>65</v>
       </c>
       <c r="B68" s="4" t="n"/>
       <c r="C68" s="4" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="9" t="inlineStr">
-        <is>
-          <t>Rebis</t>
-        </is>
+      <c r="A69" s="9" t="s">
+        <v>66</v>
       </c>
       <c r="B69" s="10" t="n"/>
       <c r="C69" s="26">
@@ -1372,10 +1557,8 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="9" t="inlineStr">
-        <is>
-          <t>Constructora</t>
-        </is>
+      <c r="A70" s="9" t="s">
+        <v>67</v>
       </c>
       <c r="B70" s="10" t="n"/>
       <c r="C70" s="26">
@@ -1384,10 +1567,8 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="inlineStr">
-        <is>
-          <t>Inversor</t>
-        </is>
+      <c r="A71" s="13" t="s">
+        <v>68</v>
       </c>
       <c r="B71" s="10" t="n"/>
       <c r="C71" s="27">
@@ -1396,10 +1577,8 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="19" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+      <c r="A72" s="19" t="s">
+        <v>69</v>
       </c>
       <c r="B72" s="20" t="n"/>
       <c r="C72" s="28">
@@ -1408,19 +1587,15 @@
       </c>
     </row>
     <row r="74" ht="17" customHeight="1">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>RESULTADO DE LA OPERACIÓN</t>
-        </is>
+      <c r="A74" s="4" t="s">
+        <v>70</v>
       </c>
       <c r="B74" s="4" t="n"/>
       <c r="C74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="inlineStr">
-        <is>
-          <t>Total costes generales</t>
-        </is>
+      <c r="A75" s="9" t="s">
+        <v>71</v>
       </c>
       <c r="B75" s="10" t="n"/>
       <c r="C75" s="18">
@@ -1429,10 +1604,8 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="9" t="inlineStr">
-        <is>
-          <t>Precio de venta estimado</t>
-        </is>
+      <c r="A76" s="9" t="s">
+        <v>7</v>
       </c>
       <c r="B76" s="10" t="n"/>
       <c r="C76" s="18">
@@ -1441,15 +1614,11 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="9" t="inlineStr">
-        <is>
-          <t>Costes de financiación a cargo de Rebis</t>
-        </is>
-      </c>
-      <c r="B77" s="17" t="inlineStr">
-        <is>
-          <t>Gastos de financiación por adquisición y por venta</t>
-        </is>
+      <c r="A77" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B77" s="17" t="s">
+        <v>73</v>
       </c>
       <c r="C77" s="18">
         <f>C34+C51</f>
@@ -1457,10 +1626,8 @@
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="22" t="inlineStr">
-        <is>
-          <t>Beneficio de la operación · sin los costes a cargo de Rebis</t>
-        </is>
+      <c r="A78" s="22" t="s">
+        <v>74</v>
       </c>
       <c r="B78" s="23" t="n"/>
       <c r="C78" s="24">
@@ -1469,30 +1636,22 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>Ganancia de la constructora</t>
-        </is>
-      </c>
-      <c r="B79" s="25" t="inlineStr">
-        <is>
-          <t>Importe fijado por Rebis; única cifra del modelo sin fórmula</t>
-        </is>
+      <c r="A79" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B79" s="25" t="s">
+        <v>76</v>
       </c>
       <c r="C79" s="7" t="n">
         <v>70846.89999999999</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="inlineStr">
-        <is>
-          <t>Honorarios de gestión de Rebis</t>
-        </is>
-      </c>
-      <c r="B80" s="17" t="inlineStr">
-        <is>
-          <t>20 % más IVA sobre el beneficio una vez deducida la constructora</t>
-        </is>
+      <c r="A80" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B80" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="C80" s="18">
         <f>ROUND((C78-C79)*0.242,2)</f>
@@ -1500,10 +1659,8 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="19" t="inlineStr">
-        <is>
-          <t>Beneficio a repartir entre los aportantes</t>
-        </is>
+      <c r="A81" s="19" t="s">
+        <v>79</v>
       </c>
       <c r="B81" s="20" t="n"/>
       <c r="C81" s="21">
@@ -1512,15 +1669,11 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="inlineStr">
-        <is>
-          <t>Ganancia del Inversor, antes de impuestos</t>
-        </is>
-      </c>
-      <c r="B82" s="17" t="inlineStr">
-        <is>
-          <t>Su porcentaje de participación sobre el beneficio a repartir</t>
-        </is>
+      <c r="A82" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>81</v>
       </c>
       <c r="C82" s="14">
         <f>ROUND(C81*C71/100,2)</f>
@@ -1528,10 +1681,8 @@
       </c>
     </row>
     <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="22" t="inlineStr">
-        <is>
-          <t>Rentabilidad del Inversor sobre el capital aportado</t>
-        </is>
+      <c r="A83" s="22" t="s">
+        <v>82</v>
       </c>
       <c r="B83" s="23" t="n"/>
       <c r="C83" s="29">
@@ -1540,15 +1691,11 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="9" t="inlineStr">
-        <is>
-          <t>Rentabilidad antes de los honorarios de Rebis</t>
-        </is>
-      </c>
-      <c r="B84" s="17" t="inlineStr">
-        <is>
-          <t>Equivalencia para comparar con operaciones sin gestión contratada</t>
-        </is>
+      <c r="A84" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B84" s="17" t="s">
+        <v>84</v>
       </c>
       <c r="C84" s="26">
         <f>(C82+C80*C71/100)/C65*100</f>
@@ -1556,65 +1703,49 @@
       </c>
     </row>
     <row r="86" ht="17" customHeight="1">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>NOTAS</t>
-        </is>
+      <c r="A86" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="B86" s="4" t="n"/>
       <c r="C86" s="4" t="n"/>
     </row>
     <row r="87" ht="12.5" customHeight="1">
-      <c r="A87" s="30" t="inlineStr">
-        <is>
-          <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes contra esas cuotas. Figura en el cuadro porque el importe debe estar disponible desde el primer día, pero el coste real de financiación de la operación es la diferencia.</t>
-        </is>
+      <c r="A87" s="30" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="88" ht="12.5" customHeight="1"/>
     <row r="89" ht="12.5" customHeight="1">
-      <c r="A89" s="30" t="inlineStr">
-        <is>
-          <t>2 · Honorarios de Rebis. Un 20 % más IVA, equivalente al 24,2 %, sobre el beneficio de la operación una vez deducida la ganancia de la constructora. Aquí Rebis no cobra comisión por la gestión de la hipoteca, porque la toma sobre su propia sociedad.</t>
-        </is>
+      <c r="A89" s="30" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="90" ht="12.5" customHeight="1"/>
     <row r="91" ht="12.5" customHeight="1">
-      <c r="A91" s="30" t="inlineStr">
-        <is>
-          <t>3 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
-        </is>
+      <c r="A91" s="30" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="92" ht="12.5" customHeight="1"/>
     <row r="93" ht="12.5" customHeight="1">
-      <c r="A93" s="30" t="inlineStr">
-        <is>
-          <t>4 · En esta opción el Inversor no figura ante el banco, no presta aval y no constituye ni administra sociedad alguna en España. La financiación bancaria, su coste y su riesgo quedan íntegramente del lado de Rebis, y por eso el apalancamiento no juega a su favor.</t>
-        </is>
+      <c r="A93" s="30" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="94" ht="12.5" customHeight="1"/>
     <row r="95" ht="12.5" customHeight="1">
-      <c r="A95" s="30" t="inlineStr">
-        <is>
-          <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
-        </is>
+      <c r="A95" s="30" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="96" ht="12.5" customHeight="1"/>
     <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="31" t="inlineStr">
-        <is>
-          <t>TRANSFORMAR CON CRITERIO.</t>
-        </is>
+      <c r="A98" s="31" t="s">
+        <v>91</v>
       </c>
       <c r="B98" s="20" t="n"/>
-      <c r="C98" s="32" t="inlineStr">
-        <is>
-          <t>rebis.com</t>
-        </is>
+      <c r="C98" s="32" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1650,17 +1781,13 @@
     <row r="1" ht="52" customHeight="1"/>
     <row r="2" ht="8" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Cash-Flow del Inversor · Opción 2</t>
-        </is>
+      <c r="A3" s="1" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Apartamento calle Ruiz Jiménez 3, Madrid.  La sociedad titular del inmueble es del Inversor, que toma la hipoteca a su nombre.  Escenario conservador.</t>
-        </is>
+      <c r="A4" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="5" ht="6" customHeight="1">
@@ -1669,19 +1796,15 @@
       <c r="C5" s="3" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>RESUMEN DE COMPRA Y VENTA</t>
-        </is>
+      <c r="A7" s="4" t="s">
+        <v>2</v>
       </c>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Precio de compra</t>
-        </is>
+      <c r="A8" s="5" t="s">
+        <v>3</v>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="n">
@@ -1689,10 +1812,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>M2 construidos</t>
-        </is>
+      <c r="A9" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="8" t="n">
@@ -1700,10 +1821,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Precio del m2 de compra</t>
-        </is>
+      <c r="A10" s="9" t="s">
+        <v>5</v>
       </c>
       <c r="B10" s="10" t="n"/>
       <c r="C10" s="11">
@@ -1712,10 +1831,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Precio del m2 de venta</t>
-        </is>
+      <c r="A11" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="12" t="n">
@@ -1723,10 +1840,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Precio de venta estimado</t>
-        </is>
+      <c r="A12" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="14">
@@ -1735,41 +1850,29 @@
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>COSTES  ·  IMPORTES CON IVA INCLUIDO</t>
-        </is>
+      <c r="A14" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="B14" s="4" t="n"/>
       <c r="C14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>ACTUACIÓN</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>CONCEPTO</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>IMPORTE</t>
-        </is>
+      <c r="A15" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Adquisición</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>Comisión inmobiliaria</t>
-        </is>
+      <c r="A16" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>13</v>
       </c>
       <c r="C16" s="18" t="n">
         <v>45375</v>
@@ -1777,10 +1880,8 @@
     </row>
     <row r="17">
       <c r="A17" s="9" t="n"/>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Honorarios legales por análisis de documentación</t>
-        </is>
+      <c r="B17" s="17" t="s">
+        <v>14</v>
       </c>
       <c r="C17" s="18" t="n">
         <v>1270.5</v>
@@ -1788,10 +1889,8 @@
     </row>
     <row r="18">
       <c r="A18" s="9" t="n"/>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>ITP · IVA · AJD</t>
-        </is>
+      <c r="B18" s="17" t="s">
+        <v>15</v>
       </c>
       <c r="C18" s="18" t="n">
         <v>30000</v>
@@ -1799,10 +1898,8 @@
     </row>
     <row r="19">
       <c r="A19" s="9" t="n"/>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>Notaría</t>
-        </is>
+      <c r="B19" s="17" t="s">
+        <v>16</v>
       </c>
       <c r="C19" s="18" t="n">
         <v>2700</v>
@@ -1810,10 +1907,8 @@
     </row>
     <row r="20">
       <c r="A20" s="9" t="n"/>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Gestoría</t>
-        </is>
+      <c r="B20" s="17" t="s">
+        <v>17</v>
       </c>
       <c r="C20" s="18" t="n">
         <v>494</v>
@@ -1821,10 +1916,8 @@
     </row>
     <row r="21">
       <c r="A21" s="9" t="n"/>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Registro de la propiedad</t>
-        </is>
+      <c r="B21" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="C21" s="18" t="n">
         <v>1600</v>
@@ -1832,20 +1925,16 @@
     </row>
     <row r="22">
       <c r="A22" s="9" t="n"/>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>IBI y tasas de basuras, proporcional 2026</t>
-        </is>
+      <c r="B22" s="17" t="s">
+        <v>19</v>
       </c>
       <c r="C22" s="18" t="n">
         <v>875</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>Total adquisición</t>
-        </is>
+      <c r="A23" s="19" t="s">
+        <v>20</v>
       </c>
       <c r="B23" s="20" t="n"/>
       <c r="C23" s="21">
@@ -1854,15 +1943,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Financiación bancaria</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>Tasación</t>
-        </is>
+      <c r="A24" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>22</v>
       </c>
       <c r="C24" s="18" t="n">
         <v>605</v>
@@ -1870,10 +1955,8 @@
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Pago otorgamiento de hipoteca (AJD)</t>
-        </is>
+      <c r="B25" s="17" t="s">
+        <v>23</v>
       </c>
       <c r="C25" s="18" t="n">
         <v>9000</v>
@@ -1881,10 +1964,8 @@
     </row>
     <row r="26">
       <c r="A26" s="9" t="n"/>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>Comisión por otorgamiento de hipoteca</t>
-        </is>
+      <c r="B26" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="C26" s="18" t="n">
         <v>2475</v>
@@ -1892,10 +1973,8 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>Contribución especial Fundación CaixaBank</t>
-        </is>
+      <c r="B27" s="17" t="s">
+        <v>25</v>
       </c>
       <c r="C27" s="18" t="n">
         <v>1200</v>
@@ -1903,10 +1982,8 @@
     </row>
     <row r="28">
       <c r="A28" s="9" t="n"/>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>Pignoración · fondo recuperable, ver nota 1</t>
-        </is>
+      <c r="B28" s="17" t="s">
+        <v>26</v>
       </c>
       <c r="C28" s="18" t="n">
         <v>38000</v>
@@ -1914,10 +1991,8 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>Gastos de hipoteca</t>
-        </is>
+      <c r="B29" s="17" t="s">
+        <v>27</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>35062.5</v>
@@ -1925,10 +2000,8 @@
     </row>
     <row r="30">
       <c r="A30" s="9" t="n"/>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>Seguro de responsabilidad civil</t>
-        </is>
+      <c r="B30" s="17" t="s">
+        <v>28</v>
       </c>
       <c r="C30" s="18" t="n">
         <v>649.51</v>
@@ -1936,10 +2009,8 @@
     </row>
     <row r="31">
       <c r="A31" s="9" t="n"/>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>Notaría</t>
-        </is>
+      <c r="B31" s="17" t="s">
+        <v>16</v>
       </c>
       <c r="C31" s="18" t="n">
         <v>2000</v>
@@ -1947,10 +2018,8 @@
     </row>
     <row r="32">
       <c r="A32" s="9" t="n"/>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>Gestoría</t>
-        </is>
+      <c r="B32" s="17" t="s">
+        <v>17</v>
       </c>
       <c r="C32" s="18" t="n">
         <v>494</v>
@@ -1958,20 +2027,16 @@
     </row>
     <row r="33">
       <c r="A33" s="9" t="n"/>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>Registro de la propiedad</t>
-        </is>
+      <c r="B33" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="C33" s="18" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>Total financiación bancaria</t>
-        </is>
+      <c r="A34" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B34" s="20" t="n"/>
       <c r="C34" s="21">
@@ -1980,15 +2045,11 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>Reforma</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>Seguro de incendio</t>
-        </is>
+      <c r="A35" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>31</v>
       </c>
       <c r="C35" s="18" t="n">
         <v>703.9400000000001</v>
@@ -1996,10 +2057,8 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="n"/>
-      <c r="B36" s="17" t="inlineStr">
-        <is>
-          <t>Asamblea para aprobación de reformas en áreas comunes</t>
-        </is>
+      <c r="B36" s="17" t="s">
+        <v>32</v>
       </c>
       <c r="C36" s="18" t="n">
         <v>150</v>
@@ -2007,10 +2066,8 @@
     </row>
     <row r="37">
       <c r="A37" s="9" t="n"/>
-      <c r="B37" s="17" t="inlineStr">
-        <is>
-          <t>Obra</t>
-        </is>
+      <c r="B37" s="17" t="s">
+        <v>33</v>
       </c>
       <c r="C37" s="18" t="n">
         <v>325000</v>
@@ -2018,10 +2075,8 @@
     </row>
     <row r="38">
       <c r="A38" s="9" t="n"/>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>Muebles</t>
-        </is>
+      <c r="B38" s="17" t="s">
+        <v>34</v>
       </c>
       <c r="C38" s="18" t="n">
         <v>30000</v>
@@ -2029,10 +2084,8 @@
     </row>
     <row r="39">
       <c r="A39" s="9" t="n"/>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>Imprevistos</t>
-        </is>
+      <c r="B39" s="17" t="s">
+        <v>35</v>
       </c>
       <c r="C39" s="18" t="n">
         <v>15000</v>
@@ -2040,10 +2093,8 @@
     </row>
     <row r="40">
       <c r="A40" s="9" t="n"/>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>Honorarios de interiorismo y arquitectura</t>
-        </is>
+      <c r="B40" s="17" t="s">
+        <v>36</v>
       </c>
       <c r="C40" s="18" t="n">
         <v>6500</v>
@@ -2051,20 +2102,16 @@
     </row>
     <row r="41">
       <c r="A41" s="9" t="n"/>
-      <c r="B41" s="17" t="inlineStr">
-        <is>
-          <t>Impuestos corrientes durante la ejecución de obra</t>
-        </is>
+      <c r="B41" s="17" t="s">
+        <v>37</v>
       </c>
       <c r="C41" s="18" t="n">
         <v>5300</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="inlineStr">
-        <is>
-          <t>Total reforma</t>
-        </is>
+      <c r="A42" s="19" t="s">
+        <v>38</v>
       </c>
       <c r="B42" s="20" t="n"/>
       <c r="C42" s="21">
@@ -2073,15 +2120,11 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="B43" s="17" t="inlineStr">
-        <is>
-          <t>Fotografía y afines</t>
-        </is>
+      <c r="A43" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>40</v>
       </c>
       <c r="C43" s="18" t="n">
         <v>900</v>
@@ -2089,10 +2132,8 @@
     </row>
     <row r="44">
       <c r="A44" s="9" t="n"/>
-      <c r="B44" s="17" t="inlineStr">
-        <is>
-          <t>IBI y tasas de basuras, proporcional 2027</t>
-        </is>
+      <c r="B44" s="17" t="s">
+        <v>41</v>
       </c>
       <c r="C44" s="18" t="n">
         <v>400</v>
@@ -2100,10 +2141,8 @@
     </row>
     <row r="45">
       <c r="A45" s="9" t="n"/>
-      <c r="B45" s="17" t="inlineStr">
-        <is>
-          <t>Comisión inmobiliaria</t>
-        </is>
+      <c r="B45" s="17" t="s">
+        <v>13</v>
       </c>
       <c r="C45" s="18">
         <f>ROUND($C$12*0.0363,2)</f>
@@ -2112,10 +2151,8 @@
     </row>
     <row r="46">
       <c r="A46" s="9" t="n"/>
-      <c r="B46" s="17" t="inlineStr">
-        <is>
-          <t>Plusvalía municipal</t>
-        </is>
+      <c r="B46" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="C46" s="18" t="n">
         <v>15000</v>
@@ -2123,10 +2160,8 @@
     </row>
     <row r="47">
       <c r="A47" s="9" t="n"/>
-      <c r="B47" s="17" t="inlineStr">
-        <is>
-          <t>Comisión por cancelación de hipoteca</t>
-        </is>
+      <c r="B47" s="17" t="s">
+        <v>45</v>
       </c>
       <c r="C47" s="18" t="n">
         <v>1237.5</v>
@@ -2134,10 +2169,8 @@
     </row>
     <row r="48">
       <c r="A48" s="9" t="n"/>
-      <c r="B48" s="17" t="inlineStr">
-        <is>
-          <t>Gestoría por cancelación de hipoteca</t>
-        </is>
+      <c r="B48" s="17" t="s">
+        <v>46</v>
       </c>
       <c r="C48" s="18" t="n">
         <v>494</v>
@@ -2145,20 +2178,16 @@
     </row>
     <row r="49">
       <c r="A49" s="9" t="n"/>
-      <c r="B49" s="17" t="inlineStr">
-        <is>
-          <t>Registro de la propiedad por cancelación</t>
-        </is>
+      <c r="B49" s="17" t="s">
+        <v>47</v>
       </c>
       <c r="C49" s="18" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="inlineStr">
-        <is>
-          <t>Total venta</t>
-        </is>
+      <c r="A50" s="19" t="s">
+        <v>43</v>
       </c>
       <c r="B50" s="20" t="n"/>
       <c r="C50" s="21">
@@ -2167,19 +2196,15 @@
       </c>
     </row>
     <row r="52" ht="17" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>CAPITAL NECESARIO PARA LA ACTUACIÓN  ·  SIN GASTOS DE VENTA</t>
-        </is>
+      <c r="A52" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="B52" s="4" t="n"/>
       <c r="C52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="inlineStr">
-        <is>
-          <t>Compra del apartamento</t>
-        </is>
+      <c r="A53" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="B53" s="10" t="n"/>
       <c r="C53" s="18">
@@ -2188,10 +2213,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>Gastos derivados de la adquisición</t>
-        </is>
+      <c r="A54" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="B54" s="10" t="n"/>
       <c r="C54" s="18">
@@ -2200,10 +2223,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
-        <is>
-          <t>Gastos de financiación bancaria</t>
-        </is>
+      <c r="A55" s="9" t="s">
+        <v>96</v>
       </c>
       <c r="B55" s="10" t="n"/>
       <c r="C55" s="18">
@@ -2212,10 +2233,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>Gastos de reforma</t>
-        </is>
+      <c r="A56" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="B56" s="10" t="n"/>
       <c r="C56" s="18">
@@ -2224,10 +2243,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="9" t="inlineStr">
-        <is>
-          <t>Fotografía y afines</t>
-        </is>
+      <c r="A57" s="9" t="s">
+        <v>40</v>
       </c>
       <c r="B57" s="10" t="n"/>
       <c r="C57" s="18" t="n">
@@ -2235,10 +2252,8 @@
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
-        <is>
-          <t>Capital necesario</t>
-        </is>
+      <c r="A58" s="22" t="s">
+        <v>53</v>
       </c>
       <c r="B58" s="23" t="n"/>
       <c r="C58" s="24">
@@ -2247,54 +2262,40 @@
       </c>
     </row>
     <row r="60" ht="17" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>APORTES DE CAPITAL</t>
-        </is>
+      <c r="A60" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="B60" s="4" t="n"/>
       <c r="C60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Aporte bancario</t>
-        </is>
-      </c>
-      <c r="B61" s="25" t="inlineStr">
-        <is>
-          <t>Hipoteca a nombre de la sociedad del Inversor, con su aval personal</t>
-        </is>
+      <c r="A61" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B61" s="25" t="s">
+        <v>98</v>
       </c>
       <c r="C61" s="7" t="n">
         <v>825000</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>Aporte de la constructora</t>
-        </is>
-      </c>
-      <c r="B62" s="25" t="inlineStr">
-        <is>
-          <t>Ejecución y financiación de obra</t>
-        </is>
+      <c r="A62" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B62" s="25" t="s">
+        <v>61</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>325000</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>Aporte del Inversor</t>
-        </is>
-      </c>
-      <c r="B63" s="17" t="inlineStr">
-        <is>
-          <t>Completa el capital necesario de la actuación</t>
-        </is>
+      <c r="A63" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B63" s="17" t="s">
+        <v>63</v>
       </c>
       <c r="C63" s="14">
         <f>C58-C61-C62</f>
@@ -2302,10 +2303,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="19" t="inlineStr">
-        <is>
-          <t>Total aportes</t>
-        </is>
+      <c r="A64" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="B64" s="20" t="n"/>
       <c r="C64" s="21">
@@ -2314,24 +2313,18 @@
       </c>
     </row>
     <row r="66" ht="17" customHeight="1">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>RESULTADO DE LA OPERACIÓN</t>
-        </is>
+      <c r="A66" s="4" t="s">
+        <v>70</v>
       </c>
       <c r="B66" s="4" t="n"/>
       <c r="C66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="9" t="inlineStr">
-        <is>
-          <t>Total costes</t>
-        </is>
-      </c>
-      <c r="B67" s="17" t="inlineStr">
-        <is>
-          <t>Sin el gasto de pignoración, que es un fondo recuperable · ver nota 1</t>
-        </is>
+      <c r="A67" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B67" s="17" t="s">
+        <v>100</v>
       </c>
       <c r="C67" s="18">
         <f>$C$8+C23+C34+C42+C50-38000</f>
@@ -2339,10 +2332,8 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="inlineStr">
-        <is>
-          <t>Precio de venta estimado</t>
-        </is>
+      <c r="A68" s="9" t="s">
+        <v>7</v>
       </c>
       <c r="B68" s="10" t="n"/>
       <c r="C68" s="18">
@@ -2351,10 +2342,8 @@
       </c>
     </row>
     <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="22" t="inlineStr">
-        <is>
-          <t>Beneficio de la operación</t>
-        </is>
+      <c r="A69" s="22" t="s">
+        <v>101</v>
       </c>
       <c r="B69" s="23" t="n"/>
       <c r="C69" s="24">
@@ -2363,30 +2352,22 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>Ganancia de la constructora</t>
-        </is>
-      </c>
-      <c r="B70" s="25" t="inlineStr">
-        <is>
-          <t>Importe fijado por Rebis; única cifra del modelo sin fórmula</t>
-        </is>
+      <c r="A70" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B70" s="25" t="s">
+        <v>76</v>
       </c>
       <c r="C70" s="7" t="n">
         <v>71924.83</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="9" t="inlineStr">
-        <is>
-          <t>Honorarios de gestión de Rebis</t>
-        </is>
-      </c>
-      <c r="B71" s="17" t="inlineStr">
-        <is>
-          <t>20 % más IVA sobre el beneficio una vez deducida la constructora</t>
-        </is>
+      <c r="A71" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B71" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="C71" s="18">
         <f>ROUND((C69-C70)*0.242,2)</f>
@@ -2394,15 +2375,11 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="9" t="inlineStr">
-        <is>
-          <t>Honorarios de Rebis por gestión y tramitación de la hipoteca</t>
-        </is>
-      </c>
-      <c r="B72" s="17" t="inlineStr">
-        <is>
-          <t>2 % más IVA sobre el importe de hipoteca concedido</t>
-        </is>
+      <c r="A72" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B72" s="17" t="s">
+        <v>103</v>
       </c>
       <c r="C72" s="18">
         <f>ROUND(C61*0.02*1.21,2)</f>
@@ -2410,15 +2387,11 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="inlineStr">
-        <is>
-          <t>Ganancia del Inversor, antes de impuestos</t>
-        </is>
-      </c>
-      <c r="B73" s="17" t="inlineStr">
-        <is>
-          <t>Recibe la totalidad del resultado restante</t>
-        </is>
+      <c r="A73" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B73" s="17" t="s">
+        <v>104</v>
       </c>
       <c r="C73" s="14">
         <f>C69-C70-C71-C72</f>
@@ -2426,10 +2399,8 @@
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="22" t="inlineStr">
-        <is>
-          <t>Rentabilidad del Inversor sobre el capital aportado</t>
-        </is>
+      <c r="A74" s="22" t="s">
+        <v>82</v>
       </c>
       <c r="B74" s="23" t="n"/>
       <c r="C74" s="29">
@@ -2438,15 +2409,11 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="inlineStr">
-        <is>
-          <t>Rentabilidad antes de los honorarios de Rebis</t>
-        </is>
-      </c>
-      <c r="B75" s="17" t="inlineStr">
-        <is>
-          <t>Equivalencia para comparar con operaciones sin gestión contratada</t>
-        </is>
+      <c r="A75" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B75" s="17" t="s">
+        <v>84</v>
       </c>
       <c r="C75" s="26">
         <f>(C73+C71+C72)/C63*100</f>
@@ -2454,65 +2421,49 @@
       </c>
     </row>
     <row r="77" ht="17" customHeight="1">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>NOTAS</t>
-        </is>
+      <c r="A77" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="B77" s="4" t="n"/>
       <c r="C77" s="4" t="n"/>
     </row>
     <row r="78" ht="12.5" customHeight="1">
-      <c r="A78" s="30" t="inlineStr">
-        <is>
-          <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes y vuelve al Inversor, de modo que aquí no se computa como coste de la operación, aunque el importe debe estar disponible desde el primer día.</t>
-        </is>
+      <c r="A78" s="30" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="79" ht="12.5" customHeight="1"/>
     <row r="80" ht="12.5" customHeight="1">
-      <c r="A80" s="30" t="inlineStr">
-        <is>
-          <t>2 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio una vez deducida la ganancia de la constructora, más un 2 % más IVA sobre el importe de hipoteca efectivamente concedido, por la gestión de la financiación y por el aval que Rebis aporta ante el banco.</t>
-        </is>
+      <c r="A80" s="30" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="81" ht="12.5" customHeight="1"/>
     <row r="82" ht="12.5" customHeight="1">
-      <c r="A82" s="30" t="inlineStr">
-        <is>
-          <t>3 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
-        </is>
+      <c r="A82" s="30" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="83" ht="12.5" customHeight="1"/>
     <row r="84" ht="12.5" customHeight="1">
-      <c r="A84" s="30" t="inlineStr">
-        <is>
-          <t>4 · En esta opción el Inversor constituye y administra la sociedad española, toma la hipoteca a su nombre y presta aval personal con su patrimonio. A cambio, el apalancamiento juega a su favor y recibe la totalidad del resultado restante, no una participación sobre él.</t>
-        </is>
+      <c r="A84" s="30" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="85" ht="12.5" customHeight="1"/>
     <row r="86" ht="12.5" customHeight="1">
-      <c r="A86" s="30" t="inlineStr">
-        <is>
-          <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
-        </is>
+      <c r="A86" s="30" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="87" ht="12.5" customHeight="1"/>
     <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="31" t="inlineStr">
-        <is>
-          <t>TRANSFORMAR CON CRITERIO.</t>
-        </is>
+      <c r="A89" s="31" t="s">
+        <v>91</v>
       </c>
       <c r="B89" s="20" t="n"/>
-      <c r="C89" s="32" t="inlineStr">
-        <is>
-          <t>rebis.com</t>
-        </is>
+      <c r="C89" s="32" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Retirar la tagline de todos los materiales
El Inversor no quiere ver «Transformar con criterio» en las piezas, así que
sale de las tres notas ejecutivas y de las dos hojas del cash-flow. Donde
estaba el claim queda la URL, que el manual ubica igual en la esquina inferior
derecha, de modo que el cierre sigue siendo el del sistema de identidad.

Se regeneran el PDF de la nota vigente y el libro, y se rehacen las dos Hojas
de cálculo de Drive. Las cifras no se mueven: 13,74 % y 22,90 %.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3Mnw54UTuPQAtnGvXf7kT
</commit_message>
<xml_diff>
--- a/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
+++ b/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="107">
   <si>
     <t>Cash-Flow del Inversor · Opción 1</t>
   </si>
@@ -289,9 +289,6 @@
   </si>
   <si>
     <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
-  </si>
-  <si>
-    <t>TRANSFORMAR CON CRITERIO.</t>
   </si>
   <si>
     <t>rebis.com</t>
@@ -351,7 +348,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;;(#,##0.00 &quot;€&quot;);—"/>
     <numFmt numFmtId="166" formatCode="0.00&quot; %&quot;"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -417,12 +414,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="FFB59169"/>
       <sz val="9"/>
     </font>
@@ -482,7 +473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -544,8 +535,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1740,12 +1730,10 @@
     </row>
     <row r="96" ht="12.5" customHeight="1"/>
     <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="31" t="s">
+      <c r="A98" s="20" t="n"/>
+      <c r="B98" s="20" t="n"/>
+      <c r="C98" s="31" t="s">
         <v>91</v>
-      </c>
-      <c r="B98" s="20" t="n"/>
-      <c r="C98" s="32" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1782,12 +1770,12 @@
     <row r="2" ht="8" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" ht="6" customHeight="1">
@@ -2197,7 +2185,7 @@
     </row>
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B52" s="4" t="n"/>
       <c r="C52" s="4" t="n"/>
@@ -2224,7 +2212,7 @@
     </row>
     <row r="55">
       <c r="A55" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B55" s="10" t="n"/>
       <c r="C55" s="18">
@@ -2270,10 +2258,10 @@
     </row>
     <row r="61">
       <c r="A61" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B61" s="25" t="s">
         <v>97</v>
-      </c>
-      <c r="B61" s="25" t="s">
-        <v>98</v>
       </c>
       <c r="C61" s="7" t="n">
         <v>825000</v>
@@ -2321,10 +2309,10 @@
     </row>
     <row r="67">
       <c r="A67" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B67" s="17" t="s">
         <v>99</v>
-      </c>
-      <c r="B67" s="17" t="s">
-        <v>100</v>
       </c>
       <c r="C67" s="18">
         <f>$C$8+C23+C34+C42+C50-38000</f>
@@ -2343,7 +2331,7 @@
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B69" s="23" t="n"/>
       <c r="C69" s="24">
@@ -2376,10 +2364,10 @@
     </row>
     <row r="72">
       <c r="A72" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B72" s="17" t="s">
         <v>102</v>
-      </c>
-      <c r="B72" s="17" t="s">
-        <v>103</v>
       </c>
       <c r="C72" s="18">
         <f>ROUND(C61*0.02*1.21,2)</f>
@@ -2391,7 +2379,7 @@
         <v>80</v>
       </c>
       <c r="B73" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C73" s="14">
         <f>C69-C70-C71-C72</f>
@@ -2429,13 +2417,13 @@
     </row>
     <row r="78" ht="12.5" customHeight="1">
       <c r="A78" s="30" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="79" ht="12.5" customHeight="1"/>
     <row r="80" ht="12.5" customHeight="1">
       <c r="A80" s="30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="81" ht="12.5" customHeight="1"/>
@@ -2447,7 +2435,7 @@
     <row r="83" ht="12.5" customHeight="1"/>
     <row r="84" ht="12.5" customHeight="1">
       <c r="A84" s="30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="85" ht="12.5" customHeight="1"/>
@@ -2458,12 +2446,10 @@
     </row>
     <row r="87" ht="12.5" customHeight="1"/>
     <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="31" t="s">
+      <c r="A89" s="20" t="n"/>
+      <c r="B89" s="20" t="n"/>
+      <c r="C89" s="31" t="s">
         <v>91</v>
-      </c>
-      <c r="B89" s="20" t="n"/>
-      <c r="C89" s="32" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reordenar notas y jerarquía de rentabilidad en el cash-flow
Ajustes pedidos por Sebastián sobre las dos hojas:

- La nota que describe la posición del Inversor pasa a encabezar el bloque,
  por delante de la pignoración. Se renumeran las cuatro y se corrige la
  referencia «ver nota 1» del cuadro de costes, que ahora apunta a la 2.
- Se invierten las dos filas de rentabilidad: primero la anterior a los
  honorarios de Rebis, que toma la negrita y el acento, y debajo la del
  Inversor sobre el capital aportado.
- En la Opción 1 la nota de honorarios se acorta. En la Opción 2 se añade que
  el Inversor responde civil, fiscal y penalmente como administrador.
- Las filas de las notas cortaban el texto: la altura pasa a calcularse según
  el largo, igual que el subtítulo de cabecera.

Las cifras no se mueven.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3Mnw54UTuPQAtnGvXf7kT
</commit_message>
<xml_diff>
--- a/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
+++ b/cashflow/Cash-Flow-Inversor-Ruiz-Jimenez-3.xlsx
@@ -96,7 +96,7 @@
     <t>Contribución especial Fundación CaixaBank</t>
   </si>
   <si>
-    <t>Pignoración · fondo recuperable, ver nota 1</t>
+    <t>Pignoración · fondo recuperable, ver nota 2</t>
   </si>
   <si>
     <t>Gastos de hipoteca</t>
@@ -264,28 +264,28 @@
     <t>Su porcentaje de participación sobre el beneficio a repartir</t>
   </si>
   <si>
+    <t>Rentabilidad antes de los honorarios de Rebis</t>
+  </si>
+  <si>
     <t>Rentabilidad del Inversor sobre el capital aportado</t>
   </si>
   <si>
-    <t>Rentabilidad antes de los honorarios de Rebis</t>
-  </si>
-  <si>
-    <t>Equivalencia para comparar con operaciones sin gestión contratada</t>
+    <t>Después de deducir los honorarios de Rebis</t>
   </si>
   <si>
     <t>NOTAS</t>
   </si>
   <si>
-    <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes contra esas cuotas. Figura en el cuadro porque el importe debe estar disponible desde el primer día, pero el coste real de financiación de la operación es la diferencia.</t>
-  </si>
-  <si>
-    <t>2 · Honorarios de Rebis. Un 20 % más IVA, equivalente al 24,2 %, sobre el beneficio de la operación una vez deducida la ganancia de la constructora. Aquí Rebis no cobra comisión por la gestión de la hipoteca, porque la toma sobre su propia sociedad.</t>
-  </si>
-  <si>
-    <t>3 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
-  </si>
-  <si>
-    <t>4 · En esta opción el Inversor no figura ante el banco, no presta aval y no constituye ni administra sociedad alguna en España. La financiación bancaria, su coste y su riesgo quedan íntegramente del lado de Rebis, y por eso el apalancamiento no juega a su favor.</t>
+    <t>1 · En esta opción el Inversor no figura ante el banco, no presta aval y no constituye ni administra sociedad alguna en España. La financiación bancaria, su coste y su riesgo quedan íntegramente del lado de Rebis, y por eso el apalancamiento no juega a su favor.</t>
+  </si>
+  <si>
+    <t>2 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes contra esas cuotas. Figura en el cuadro porque el importe debe estar disponible desde el primer día, pero el coste real de financiación de la operación es la diferencia.</t>
+  </si>
+  <si>
+    <t>3 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio de la operación. Rebis no cobra comisión por la gestión de la hipoteca.</t>
+  </si>
+  <si>
+    <t>4 · Rentabilidad. La cifra es posterior a los honorarios de Rebis y anterior a los impuestos del Inversor. El impuesto a la renta queda fuera del modelo, como en cualquier inversión, y depende de la residencia fiscal de cada aportante.</t>
   </si>
   <si>
     <t>Las celdas con fondo cerámica son los datos de entrada del modelo: precio de compra, metros construidos, precio del m2 de venta y los aportes. El resto del cuadro se recalcula solo.</t>
@@ -315,7 +315,7 @@
     <t>Total costes</t>
   </si>
   <si>
-    <t>Sin el gasto de pignoración, que es un fondo recuperable · ver nota 1</t>
+    <t>Sin el gasto de pignoración, que es un fondo recuperable · ver nota 2</t>
   </si>
   <si>
     <t>Beneficio de la operación</t>
@@ -330,13 +330,13 @@
     <t>Recibe la totalidad del resultado restante</t>
   </si>
   <si>
-    <t>1 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes y vuelve al Inversor, de modo que aquí no se computa como coste de la operación, aunque el importe debe estar disponible desde el primer día.</t>
-  </si>
-  <si>
-    <t>2 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio una vez deducida la ganancia de la constructora, más un 2 % más IVA sobre el importe de hipoteca efectivamente concedido, por la gestión de la financiación y por el aval que Rebis aporta ante el banco.</t>
-  </si>
-  <si>
-    <t>4 · En esta opción el Inversor constituye y administra la sociedad española, toma la hipoteca a su nombre y presta aval personal con su patrimonio. A cambio, el apalancamiento juega a su favor y recibe la totalidad del resultado restante, no una participación sobre él.</t>
+    <t>1 · En esta opción el Inversor constituye y administra la sociedad española, toma la hipoteca a su nombre, presta aval personal con su patrimonio y responde civil, fiscal y penalmente como administrador. A cambio, el apalancamiento juega a su favor y recibe la totalidad del resultado restante, no una participación sobre él.</t>
+  </si>
+  <si>
+    <t>2 · Pignoración. Los 38.000 € no son un gasto: son un fondo que el banco retiene en garantía de unas 13 cuotas del período de carencia, durante el cual no se amortiza capital y solo se pagan intereses. El fondo se libera mes a mes y vuelve al Inversor, de modo que aquí no se computa como coste de la operación, aunque el importe debe estar disponible desde el primer día.</t>
+  </si>
+  <si>
+    <t>3 · Honorarios de Rebis. Un 20 % más IVA sobre el beneficio una vez deducida la ganancia de la constructora, más un 2 % más IVA sobre el importe de hipoteca efectivamente concedido, por la gestión de la financiación y por el aval que Rebis aporta ante el banco.</t>
   </si>
 </sst>
 </file>
@@ -978,7 +978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" ht="26" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1676,8 +1676,8 @@
       </c>
       <c r="B83" s="23" t="n"/>
       <c r="C83" s="29">
-        <f>C82/C65*100</f>
-        <v>13.740679563</v>
+        <f>(C82+C80*C71/100)/C65*100</f>
+        <v>18.1275458581</v>
       </c>
     </row>
     <row r="84">
@@ -1688,8 +1688,8 @@
         <v>84</v>
       </c>
       <c r="C84" s="26">
-        <f>(C82+C80*C71/100)/C65*100</f>
-        <v>18.1275458581</v>
+        <f>C82/C65*100</f>
+        <v>13.740679563</v>
       </c>
     </row>
     <row r="86" ht="17" customHeight="1">
@@ -1699,36 +1699,36 @@
       <c r="B86" s="4" t="n"/>
       <c r="C86" s="4" t="n"/>
     </row>
-    <row r="87" ht="12.5" customHeight="1">
+    <row r="87" ht="18.5" customHeight="1">
       <c r="A87" s="30" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="88" ht="12.5" customHeight="1"/>
-    <row r="89" ht="12.5" customHeight="1">
+    <row r="88" ht="18.5" customHeight="1"/>
+    <row r="89" ht="24" customHeight="1">
       <c r="A89" s="30" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="90" ht="12.5" customHeight="1"/>
-    <row r="91" ht="12.5" customHeight="1">
+    <row r="90" ht="24" customHeight="1"/>
+    <row r="91" ht="13" customHeight="1">
       <c r="A91" s="30" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="92" ht="12.5" customHeight="1"/>
-    <row r="93" ht="12.5" customHeight="1">
+    <row r="92" ht="13" customHeight="1"/>
+    <row r="93" ht="13" customHeight="1">
       <c r="A93" s="30" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="94" ht="12.5" customHeight="1"/>
-    <row r="95" ht="12.5" customHeight="1">
+    <row r="94" ht="13" customHeight="1"/>
+    <row r="95" ht="13" customHeight="1">
       <c r="A95" s="30" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="96" ht="12.5" customHeight="1"/>
+    <row r="96" ht="13" customHeight="1"/>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="20" t="n"/>
       <c r="B98" s="20" t="n"/>
@@ -1773,7 +1773,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" ht="26" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>93</v>
       </c>
@@ -2392,8 +2392,8 @@
       </c>
       <c r="B74" s="23" t="n"/>
       <c r="C74" s="29">
-        <f>C73/C63*100</f>
-        <v>22.9033402264</v>
+        <f>(C73+C71+C72)/C63*100</f>
+        <v>33.1218522568</v>
       </c>
     </row>
     <row r="75">
@@ -2404,8 +2404,8 @@
         <v>84</v>
       </c>
       <c r="C75" s="26">
-        <f>(C73+C71+C72)/C63*100</f>
-        <v>33.1218522568</v>
+        <f>C73/C63*100</f>
+        <v>22.9033402264</v>
       </c>
     </row>
     <row r="77" ht="17" customHeight="1">
@@ -2415,36 +2415,36 @@
       <c r="B77" s="4" t="n"/>
       <c r="C77" s="4" t="n"/>
     </row>
-    <row r="78" ht="12.5" customHeight="1">
+    <row r="78" ht="18.5" customHeight="1">
       <c r="A78" s="30" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="79" ht="12.5" customHeight="1"/>
-    <row r="80" ht="12.5" customHeight="1">
+    <row r="79" ht="18.5" customHeight="1"/>
+    <row r="80" ht="24" customHeight="1">
       <c r="A80" s="30" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="81" ht="12.5" customHeight="1"/>
-    <row r="82" ht="12.5" customHeight="1">
+    <row r="81" ht="24" customHeight="1"/>
+    <row r="82" ht="18.5" customHeight="1">
       <c r="A82" s="30" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="83" ht="12.5" customHeight="1"/>
-    <row r="84" ht="12.5" customHeight="1">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="83" ht="18.5" customHeight="1"/>
+    <row r="84" ht="13" customHeight="1">
       <c r="A84" s="30" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="85" ht="12.5" customHeight="1"/>
-    <row r="86" ht="12.5" customHeight="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="85" ht="13" customHeight="1"/>
+    <row r="86" ht="13" customHeight="1">
       <c r="A86" s="30" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="87" ht="12.5" customHeight="1"/>
+    <row r="87" ht="13" customHeight="1"/>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="20" t="n"/>
       <c r="B89" s="20" t="n"/>

</xml_diff>